<commit_message>
data with steam load and changes in the code
</commit_message>
<xml_diff>
--- a/hourly datasets/PlantID_year-4final.xlsx
+++ b/hourly datasets/PlantID_year-4final.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C145"/>
+  <dimension ref="A1:C147"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -931,1101 +931,1123 @@
     </row>
     <row r="46">
       <c r="A46" t="n">
-        <v>3140</v>
+        <v>3152</v>
       </c>
       <c r="B46" t="n">
-        <v>0.3608692261421088</v>
+        <v>0.56709112999304</v>
       </c>
       <c r="C46" t="n">
-        <v>0.3227148099598149</v>
+        <v>0.4966341528697863</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="n">
-        <v>3131</v>
+        <v>3148</v>
       </c>
       <c r="B47" t="n">
-        <v>0.3560229317470405</v>
+        <v>0.3223629328616754</v>
       </c>
       <c r="C47" t="n">
-        <v>0.3031239627150191</v>
+        <v>0.2891267738276887</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="n">
-        <v>3118</v>
+        <v>3140</v>
       </c>
       <c r="B48" t="n">
-        <v>0.3644217095493537</v>
+        <v>0.3608692261421088</v>
       </c>
       <c r="C48" t="n">
-        <v>0.3072503879074647</v>
+        <v>0.3227148099598149</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="n">
-        <v>3113</v>
+        <v>3131</v>
       </c>
       <c r="B49" t="n">
-        <v>0.3870997564043199</v>
+        <v>0.3560229317470405</v>
       </c>
       <c r="C49" t="n">
-        <v>0.1611534039363451</v>
+        <v>0.3031239627150191</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="n">
-        <v>2878</v>
+        <v>3118</v>
       </c>
       <c r="B50" t="n">
-        <v>0.3731426453658845</v>
+        <v>0.3644217095493537</v>
       </c>
       <c r="C50" t="n">
-        <v>0.3766221542515145</v>
+        <v>0.3072503879074647</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="n">
-        <v>2876</v>
+        <v>3113</v>
       </c>
       <c r="B51" t="n">
-        <v>0.3714344482390222</v>
+        <v>0.3870997564043199</v>
       </c>
       <c r="C51" t="n">
-        <v>0.3753520536981952</v>
+        <v>0.1611534039363451</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="n">
-        <v>2872</v>
+        <v>2878</v>
       </c>
       <c r="B52" t="n">
-        <v>0.3816908723548493</v>
+        <v>0.3731426453658845</v>
       </c>
       <c r="C52" t="n">
-        <v>0.3822033877803676</v>
+        <v>0.3766221542515145</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="n">
-        <v>2866</v>
+        <v>2876</v>
       </c>
       <c r="B53" t="n">
-        <v>0.348565769238066</v>
+        <v>0.3714344482390222</v>
       </c>
       <c r="C53" t="n">
-        <v>0.2695885480183995</v>
+        <v>0.3753520536981952</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="n">
-        <v>2861</v>
+        <v>2872</v>
       </c>
       <c r="B54" t="n">
-        <v>0.3412229408875688</v>
+        <v>0.3816908723548493</v>
       </c>
       <c r="C54" t="n">
-        <v>0.2364963427400908</v>
+        <v>0.3822033877803676</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="n">
-        <v>2857</v>
+        <v>2866</v>
       </c>
       <c r="B55" t="n">
-        <v>0.3824294957911895</v>
+        <v>0.3485492409531383</v>
       </c>
       <c r="C55" t="n">
-        <v>0.2678828051140654</v>
+        <v>0.2695872999860202</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="n">
-        <v>2850</v>
+        <v>2861</v>
       </c>
       <c r="B56" t="n">
-        <v>0.3579566481111134</v>
+        <v>0.3412229408875688</v>
       </c>
       <c r="C56" t="n">
-        <v>0.3558764325899996</v>
+        <v>0.2364963427400908</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="n">
-        <v>2843</v>
+        <v>2857</v>
       </c>
       <c r="B57" t="n">
-        <v>0.3135601166183295</v>
+        <v>0.3824294957911895</v>
       </c>
       <c r="C57" t="n">
-        <v>0.1829303134549639</v>
+        <v>0.2678828051140654</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="n">
-        <v>2840</v>
+        <v>2850</v>
       </c>
       <c r="B58" t="n">
-        <v>0.3621813144046631</v>
+        <v>0.3579566481111134</v>
       </c>
       <c r="C58" t="n">
-        <v>0.3094982158190912</v>
+        <v>0.3558764325899996</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="n">
-        <v>2838</v>
+        <v>2843</v>
       </c>
       <c r="B59" t="n">
-        <v>2.604304879396142</v>
+        <v>0.3135601166183295</v>
       </c>
       <c r="C59" t="n">
-        <v>0.08878850733104968</v>
+        <v>0.1829303134549639</v>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="n">
-        <v>2837</v>
+        <v>2840</v>
       </c>
       <c r="B60" t="n">
-        <v>0.3791077949882992</v>
+        <v>0.3621813144046631</v>
       </c>
       <c r="C60" t="n">
-        <v>0.2795475628018562</v>
+        <v>0.3094982158190912</v>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="n">
-        <v>2836</v>
+        <v>2838</v>
       </c>
       <c r="B61" t="n">
-        <v>0.3497206129677597</v>
+        <v>2.604304879396142</v>
       </c>
       <c r="C61" t="n">
-        <v>0.1265192524180493</v>
+        <v>0.08878850733104968</v>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="n">
-        <v>2835</v>
+        <v>2837</v>
       </c>
       <c r="B62" t="n">
-        <v>0.4834529714480031</v>
+        <v>0.3791077949882992</v>
       </c>
       <c r="C62" t="n">
-        <v>0.3225488769773652</v>
+        <v>0.2795475628018562</v>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="n">
-        <v>2832</v>
+        <v>2836</v>
       </c>
       <c r="B63" t="n">
-        <v>0.3332437817966996</v>
+        <v>0.3497206129677597</v>
       </c>
       <c r="C63" t="n">
-        <v>0.3207110353591079</v>
+        <v>0.1265192524180493</v>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="n">
-        <v>2830</v>
+        <v>2835</v>
       </c>
       <c r="B64" t="n">
-        <v>0.35594901205693</v>
+        <v>0.4834529714480031</v>
       </c>
       <c r="C64" t="n">
-        <v>0.3267552515939188</v>
+        <v>0.3225488769773652</v>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="n">
-        <v>2828</v>
+        <v>2832</v>
       </c>
       <c r="B65" t="n">
-        <v>0.3579022467365578</v>
+        <v>0.3332437817966996</v>
       </c>
       <c r="C65" t="n">
-        <v>0.2415511146651811</v>
+        <v>0.3207110353591079</v>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="n">
-        <v>2594</v>
+        <v>2830</v>
       </c>
       <c r="B66" t="n">
-        <v>0.3870171691183409</v>
+        <v>0.35594901205693</v>
       </c>
       <c r="C66" t="n">
-        <v>0.2421771107376635</v>
+        <v>0.3267552515939188</v>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="n">
-        <v>2554</v>
+        <v>2828</v>
       </c>
       <c r="B67" t="n">
-        <v>0.4007194333090533</v>
+        <v>0.3579022467365578</v>
       </c>
       <c r="C67" t="n">
-        <v>0.3033797962161246</v>
+        <v>0.2415511146651811</v>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="n">
-        <v>2527</v>
+        <v>2594</v>
       </c>
       <c r="B68" t="n">
-        <v>0.3749280884543377</v>
+        <v>0.3870171691183409</v>
       </c>
       <c r="C68" t="n">
-        <v>0.2527244504894599</v>
+        <v>0.2421771107376635</v>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="n">
-        <v>2517</v>
+        <v>2554</v>
       </c>
       <c r="B69" t="n">
-        <v>0.3698113610556444</v>
+        <v>0.4007194333090533</v>
       </c>
       <c r="C69" t="n">
-        <v>0.2735154161934025</v>
+        <v>0.3033797962161246</v>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="n">
-        <v>2516</v>
+        <v>2535</v>
       </c>
       <c r="B70" t="n">
-        <v>0.3510069218524295</v>
+        <v>0.3190059885038629</v>
       </c>
       <c r="C70" t="n">
-        <v>0.2874998238539221</v>
+        <v>0.3150614873796498</v>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="n">
-        <v>2378</v>
+        <v>2527</v>
       </c>
       <c r="B71" t="n">
-        <v>0.4021462501649309</v>
+        <v>0.3749280884543377</v>
       </c>
       <c r="C71" t="n">
-        <v>0.3015352332040474</v>
+        <v>0.2527244504894599</v>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="n">
-        <v>2364</v>
+        <v>2517</v>
       </c>
       <c r="B72" t="n">
-        <v>0.360039719292635</v>
+        <v>0.3698113610556444</v>
       </c>
       <c r="C72" t="n">
-        <v>0.2994914749965086</v>
+        <v>0.2735154161934025</v>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="n">
-        <v>2168</v>
+        <v>2516</v>
       </c>
       <c r="B73" t="n">
-        <v>0.3576921311909673</v>
+        <v>0.3510069218524295</v>
       </c>
       <c r="C73" t="n">
-        <v>0.2950274441264135</v>
+        <v>0.2874998238539221</v>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="n">
-        <v>2167</v>
+        <v>2378</v>
       </c>
       <c r="B74" t="n">
-        <v>0.3582742137454484</v>
+        <v>0.4021462501649309</v>
       </c>
       <c r="C74" t="n">
-        <v>0.2822159719845896</v>
+        <v>0.3015352332040474</v>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="n">
-        <v>2161</v>
+        <v>2364</v>
       </c>
       <c r="B75" t="n">
-        <v>0.3682798786874736</v>
+        <v>0.360039719292635</v>
       </c>
       <c r="C75" t="n">
-        <v>0.2833219127598758</v>
+        <v>0.2994914749965086</v>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="n">
-        <v>2107</v>
+        <v>2168</v>
       </c>
       <c r="B76" t="n">
-        <v>0.3454269318322105</v>
+        <v>0.3576921311909673</v>
       </c>
       <c r="C76" t="n">
-        <v>0.1767351408063946</v>
+        <v>0.2950274441264135</v>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="n">
-        <v>2104</v>
+        <v>2167</v>
       </c>
       <c r="B77" t="n">
-        <v>0.3323239723586519</v>
+        <v>0.3582742137454484</v>
       </c>
       <c r="C77" t="n">
-        <v>0.3007119184708865</v>
+        <v>0.2822159719845896</v>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="n">
-        <v>2103</v>
+        <v>2161</v>
       </c>
       <c r="B78" t="n">
-        <v>0.3408509660557938</v>
+        <v>0.3682798786874736</v>
       </c>
       <c r="C78" t="n">
-        <v>0.3350687471037519</v>
+        <v>0.2833219127598758</v>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="n">
-        <v>2094</v>
+        <v>2107</v>
       </c>
       <c r="B79" t="n">
-        <v>0.3350319360420932</v>
+        <v>0.3454269318322105</v>
       </c>
       <c r="C79" t="n">
-        <v>0.2990874840283987</v>
+        <v>0.1767351408063946</v>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="n">
-        <v>2080</v>
+        <v>2104</v>
       </c>
       <c r="B80" t="n">
-        <v>0.2984522925637598</v>
+        <v>0.3323239723586519</v>
       </c>
       <c r="C80" t="n">
-        <v>0.2253424006096986</v>
+        <v>0.3007119184708865</v>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="n">
-        <v>2079</v>
+        <v>2103</v>
       </c>
       <c r="B81" t="n">
-        <v>0.4920055140540828</v>
+        <v>0.3408509660557938</v>
       </c>
       <c r="C81" t="n">
-        <v>0.332831843028485</v>
+        <v>0.3350687471037519</v>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="n">
-        <v>2076</v>
+        <v>2094</v>
       </c>
       <c r="B82" t="n">
-        <v>0.4048803021393707</v>
+        <v>0.3350319360420932</v>
       </c>
       <c r="C82" t="n">
-        <v>0.2257864059858031</v>
+        <v>0.2990874840283987</v>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="n">
-        <v>2049</v>
+        <v>2080</v>
       </c>
       <c r="B83" t="n">
-        <v>0.3613718015950349</v>
+        <v>0.2984522925637598</v>
       </c>
       <c r="C83" t="n">
-        <v>0.2986295917733249</v>
+        <v>0.2253424006096986</v>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="n">
-        <v>1912</v>
+        <v>2079</v>
       </c>
       <c r="B84" t="n">
-        <v>0.5213840596956788</v>
+        <v>0.4920055140540828</v>
       </c>
       <c r="C84" t="n">
-        <v>0.1869888518525323</v>
+        <v>0.332831843028485</v>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="n">
-        <v>1723</v>
+        <v>2076</v>
       </c>
       <c r="B85" t="n">
-        <v>0.3716312694452902</v>
+        <v>0.4048803021393707</v>
       </c>
       <c r="C85" t="n">
-        <v>0.2806189290612324</v>
+        <v>0.2257864059858031</v>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="n">
-        <v>1720</v>
+        <v>2049</v>
       </c>
       <c r="B86" t="n">
-        <v>0.3744743974591479</v>
+        <v>0.3613718015950349</v>
       </c>
       <c r="C86" t="n">
-        <v>0.189875698102339</v>
+        <v>0.2986295917733249</v>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="n">
-        <v>1710</v>
+        <v>1912</v>
       </c>
       <c r="B87" t="n">
-        <v>0.3940655355512691</v>
+        <v>0.5213840596956788</v>
       </c>
       <c r="C87" t="n">
-        <v>0.3432023137636835</v>
+        <v>0.1869888518525323</v>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="n">
-        <v>1702</v>
+        <v>1723</v>
       </c>
       <c r="B88" t="n">
-        <v>0.3729988994955625</v>
+        <v>0.3716312694452902</v>
       </c>
       <c r="C88" t="n">
-        <v>0.376989498882803</v>
+        <v>0.2806189290612324</v>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="n">
-        <v>1619</v>
+        <v>1720</v>
       </c>
       <c r="B89" t="n">
-        <v>0.4822602500308986</v>
+        <v>0.3744743974591479</v>
       </c>
       <c r="C89" t="n">
-        <v>0.3129963387890729</v>
+        <v>0.189875698102339</v>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="n">
-        <v>1606</v>
+        <v>1710</v>
       </c>
       <c r="B90" t="n">
-        <v>0.4111931147911536</v>
+        <v>0.3940655355512691</v>
       </c>
       <c r="C90" t="n">
-        <v>0.2576834094500449</v>
+        <v>0.3432023137636835</v>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="n">
-        <v>1573</v>
+        <v>1702</v>
       </c>
       <c r="B91" t="n">
-        <v>0.3850465353245314</v>
+        <v>0.3729988994955625</v>
       </c>
       <c r="C91" t="n">
-        <v>0.318426680414835</v>
+        <v>0.376989498882803</v>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="n">
-        <v>1571</v>
+        <v>1619</v>
       </c>
       <c r="B92" t="n">
-        <v>0.3647835277017356</v>
+        <v>0.4822602500308986</v>
       </c>
       <c r="C92" t="n">
-        <v>0.3263599274711367</v>
+        <v>0.3129963387890729</v>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="n">
-        <v>1570</v>
+        <v>1606</v>
       </c>
       <c r="B93" t="n">
-        <v>0.3309031813868305</v>
+        <v>0.4111931147911536</v>
       </c>
       <c r="C93" t="n">
-        <v>0.2175192469636241</v>
+        <v>0.2576834094500449</v>
       </c>
     </row>
     <row r="94">
       <c r="A94" t="n">
-        <v>1552</v>
+        <v>1573</v>
       </c>
       <c r="B94" t="n">
-        <v>0.3189135236987325</v>
+        <v>0.3850465353245314</v>
       </c>
       <c r="C94" t="n">
-        <v>0.1819597408102214</v>
+        <v>0.318426680414835</v>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="n">
-        <v>1384</v>
+        <v>1571</v>
       </c>
       <c r="B95" t="n">
-        <v>0.3709580368288992</v>
+        <v>0.3647835277017356</v>
       </c>
       <c r="C95" t="n">
-        <v>0.3539739019315459</v>
+        <v>0.3263599274711367</v>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="n">
-        <v>1382</v>
+        <v>1570</v>
       </c>
       <c r="B96" t="n">
-        <v>0.3091456705991906</v>
+        <v>0.3309031813868305</v>
       </c>
       <c r="C96" t="n">
-        <v>0.06304002232048303</v>
+        <v>0.2175192469636241</v>
       </c>
     </row>
     <row r="97">
       <c r="A97" t="n">
-        <v>1381</v>
+        <v>1552</v>
       </c>
       <c r="B97" t="n">
-        <v>0.3561356106057925</v>
+        <v>0.3189135236987325</v>
       </c>
       <c r="C97" t="n">
-        <v>0.3316217407851156</v>
+        <v>0.1819597408102214</v>
       </c>
     </row>
     <row r="98">
       <c r="A98" t="n">
-        <v>1379</v>
+        <v>1384</v>
       </c>
       <c r="B98" t="n">
-        <v>0.2602492216789122</v>
+        <v>0.3709580368288992</v>
       </c>
       <c r="C98" t="n">
-        <v>0.2192747352870803</v>
+        <v>0.3539739019315459</v>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="n">
-        <v>1378</v>
+        <v>1382</v>
       </c>
       <c r="B99" t="n">
-        <v>0.5667705677812378</v>
+        <v>0.3091456705991906</v>
       </c>
       <c r="C99" t="n">
-        <v>0.1794564314696095</v>
+        <v>0.06304002232048303</v>
       </c>
     </row>
     <row r="100">
       <c r="A100" t="n">
-        <v>1374</v>
+        <v>1381</v>
       </c>
       <c r="B100" t="n">
-        <v>0.3139419296879841</v>
+        <v>0.3561356106057925</v>
       </c>
       <c r="C100" t="n">
-        <v>0.1583872230727588</v>
+        <v>0.3316217407851156</v>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="n">
-        <v>1357</v>
+        <v>1379</v>
       </c>
       <c r="B101" t="n">
-        <v>0.3147888834803775</v>
+        <v>0.2602492216789122</v>
       </c>
       <c r="C101" t="n">
-        <v>0.2211515454740631</v>
+        <v>0.2192747352870803</v>
       </c>
     </row>
     <row r="102">
       <c r="A102" t="n">
-        <v>1356</v>
+        <v>1378</v>
       </c>
       <c r="B102" t="n">
-        <v>0.404001646717537</v>
+        <v>0.5667705677812378</v>
       </c>
       <c r="C102" t="n">
-        <v>0.3195114566958964</v>
+        <v>0.1794564314696095</v>
       </c>
     </row>
     <row r="103">
       <c r="A103" t="n">
-        <v>1355</v>
+        <v>1374</v>
       </c>
       <c r="B103" t="n">
-        <v>0.3487187858547596</v>
+        <v>0.3139419296879841</v>
       </c>
       <c r="C103" t="n">
-        <v>0.3040080299850326</v>
+        <v>0.1583872230727588</v>
       </c>
     </row>
     <row r="104">
       <c r="A104" t="n">
-        <v>1295</v>
+        <v>1357</v>
       </c>
       <c r="B104" t="n">
-        <v>2.05177247605194</v>
+        <v>0.3147888834803775</v>
       </c>
       <c r="C104" t="n">
-        <v>0.2749952266905087</v>
+        <v>0.2211515454740631</v>
       </c>
     </row>
     <row r="105">
       <c r="A105" t="n">
-        <v>1241</v>
+        <v>1356</v>
       </c>
       <c r="B105" t="n">
-        <v>0.390066111243477</v>
+        <v>0.404001646717537</v>
       </c>
       <c r="C105" t="n">
-        <v>0.2325610711514961</v>
+        <v>0.3195114566958964</v>
       </c>
     </row>
     <row r="106">
       <c r="A106" t="n">
-        <v>1104</v>
+        <v>1355</v>
       </c>
       <c r="B106" t="n">
-        <v>0.3260176678836244</v>
+        <v>0.3487187858547596</v>
       </c>
       <c r="C106" t="n">
-        <v>0.1521048992032321</v>
+        <v>0.3040080299850326</v>
       </c>
     </row>
     <row r="107">
       <c r="A107" t="n">
-        <v>1081</v>
+        <v>1295</v>
       </c>
       <c r="B107" t="n">
-        <v>0.5507934642717458</v>
+        <v>2.05177247605194</v>
       </c>
       <c r="C107" t="n">
-        <v>0.342973349438488</v>
+        <v>0.2749952266905087</v>
       </c>
     </row>
     <row r="108">
       <c r="A108" t="n">
-        <v>1073</v>
+        <v>1241</v>
       </c>
       <c r="B108" t="n">
-        <v>0.3825847251278167</v>
+        <v>0.390066111243477</v>
       </c>
       <c r="C108" t="n">
-        <v>0.1028952642360957</v>
+        <v>0.2325610711514961</v>
       </c>
     </row>
     <row r="109">
       <c r="A109" t="n">
-        <v>1048</v>
+        <v>1104</v>
       </c>
       <c r="B109" t="n">
-        <v>0.3474893300106217</v>
+        <v>0.3260176678836244</v>
       </c>
       <c r="C109" t="n">
-        <v>0.3008380441315619</v>
+        <v>0.1521048992032321</v>
       </c>
     </row>
     <row r="110">
       <c r="A110" t="n">
-        <v>1043</v>
+        <v>1081</v>
       </c>
       <c r="B110" t="n">
-        <v>0.3453720536206965</v>
+        <v>0.5507934642717458</v>
       </c>
       <c r="C110" t="n">
-        <v>0.3010690731983817</v>
+        <v>0.342973349438488</v>
       </c>
     </row>
     <row r="111">
       <c r="A111" t="n">
-        <v>1012</v>
+        <v>1048</v>
       </c>
       <c r="B111" t="n">
-        <v>0.3046535248917526</v>
+        <v>0.3474893300106217</v>
       </c>
       <c r="C111" t="n">
-        <v>0.2827103819132206</v>
+        <v>0.3008380441315619</v>
       </c>
     </row>
     <row r="112">
       <c r="A112" t="n">
-        <v>1010</v>
+        <v>1043</v>
       </c>
       <c r="B112" t="n">
-        <v>0.5023904058892911</v>
+        <v>0.3453720536206965</v>
       </c>
       <c r="C112" t="n">
-        <v>0.2494889898667585</v>
+        <v>0.3010690731983817</v>
       </c>
     </row>
     <row r="113">
       <c r="A113" t="n">
-        <v>1008</v>
+        <v>1012</v>
       </c>
       <c r="B113" t="n">
-        <v>0.2836355858900913</v>
+        <v>0.3046535248917526</v>
       </c>
       <c r="C113" t="n">
-        <v>0.2248366001098001</v>
+        <v>0.2827103819132206</v>
       </c>
     </row>
     <row r="114">
       <c r="A114" t="n">
-        <v>1001</v>
+        <v>1010</v>
       </c>
       <c r="B114" t="n">
-        <v>0.3373614043107674</v>
+        <v>0.5023904058892911</v>
       </c>
       <c r="C114" t="n">
-        <v>0.2351861726741784</v>
+        <v>0.2494889898667585</v>
       </c>
     </row>
     <row r="115">
       <c r="A115" t="n">
-        <v>997</v>
+        <v>1008</v>
       </c>
       <c r="B115" t="n">
-        <v>0.3154158372992738</v>
+        <v>0.2836355858900913</v>
       </c>
       <c r="C115" t="n">
-        <v>0.1414537313146478</v>
+        <v>0.2248366001098001</v>
       </c>
     </row>
     <row r="116">
       <c r="A116" t="n">
-        <v>995</v>
+        <v>1001</v>
       </c>
       <c r="B116" t="n">
-        <v>0.3341057713080128</v>
+        <v>0.3373614043107674</v>
       </c>
       <c r="C116" t="n">
-        <v>0.1099034620669631</v>
+        <v>0.2351861726741784</v>
       </c>
     </row>
     <row r="117">
       <c r="A117" t="n">
-        <v>994</v>
+        <v>997</v>
       </c>
       <c r="B117" t="n">
-        <v>0.3193461637203914</v>
+        <v>0.3154158372992738</v>
       </c>
       <c r="C117" t="n">
-        <v>0.3002334817384795</v>
+        <v>0.1414537313146478</v>
       </c>
     </row>
     <row r="118">
       <c r="A118" t="n">
-        <v>991</v>
+        <v>995</v>
       </c>
       <c r="B118" t="n">
-        <v>0.377597647224074</v>
+        <v>0.3341057713080128</v>
       </c>
       <c r="C118" t="n">
-        <v>0.3028253148388222</v>
+        <v>0.1099034620669631</v>
       </c>
     </row>
     <row r="119">
       <c r="A119" t="n">
-        <v>990</v>
+        <v>994</v>
       </c>
       <c r="B119" t="n">
-        <v>0.3200383648458848</v>
+        <v>0.3193461637203914</v>
       </c>
       <c r="C119" t="n">
-        <v>0.3007083663699309</v>
+        <v>0.3002334817384795</v>
       </c>
     </row>
     <row r="120">
       <c r="A120" t="n">
-        <v>988</v>
+        <v>991</v>
       </c>
       <c r="B120" t="n">
-        <v>0.4369362396923436</v>
+        <v>0.377597647224074</v>
       </c>
       <c r="C120" t="n">
-        <v>0.219423550284241</v>
+        <v>0.3028253148388222</v>
       </c>
     </row>
     <row r="121">
       <c r="A121" t="n">
-        <v>983</v>
+        <v>990</v>
       </c>
       <c r="B121" t="n">
-        <v>0.3643001584047057</v>
+        <v>0.3200383648458848</v>
       </c>
       <c r="C121" t="n">
-        <v>0.3554259716397997</v>
+        <v>0.3007083663699309</v>
       </c>
     </row>
     <row r="122">
       <c r="A122" t="n">
-        <v>897</v>
+        <v>988</v>
       </c>
       <c r="B122" t="n">
-        <v>0.3753025580695051</v>
+        <v>0.4369362396923436</v>
       </c>
       <c r="C122" t="n">
-        <v>0.2080688625334745</v>
+        <v>0.219423550284241</v>
       </c>
     </row>
     <row r="123">
       <c r="A123" t="n">
-        <v>892</v>
+        <v>983</v>
       </c>
       <c r="B123" t="n">
-        <v>0.3423287839730054</v>
+        <v>0.3643001584047057</v>
       </c>
       <c r="C123" t="n">
-        <v>0.176354625030066</v>
+        <v>0.3554259716397997</v>
       </c>
     </row>
     <row r="124">
       <c r="A124" t="n">
-        <v>889</v>
+        <v>897</v>
       </c>
       <c r="B124" t="n">
-        <v>0.368209472500456</v>
+        <v>0.3753025580695051</v>
       </c>
       <c r="C124" t="n">
-        <v>0.2468045397430277</v>
+        <v>0.2080688625334745</v>
       </c>
     </row>
     <row r="125">
       <c r="A125" t="n">
-        <v>887</v>
+        <v>892</v>
       </c>
       <c r="B125" t="n">
-        <v>0.3217583741703381</v>
+        <v>0.3423287839730054</v>
       </c>
       <c r="C125" t="n">
-        <v>0.3209856327912293</v>
+        <v>0.176354625030066</v>
       </c>
     </row>
     <row r="126">
       <c r="A126" t="n">
-        <v>876</v>
+        <v>889</v>
       </c>
       <c r="B126" t="n">
-        <v>0.3490808065648447</v>
+        <v>0.368209472500456</v>
       </c>
       <c r="C126" t="n">
-        <v>0.1408378652040445</v>
+        <v>0.2468045397430277</v>
       </c>
     </row>
     <row r="127">
       <c r="A127" t="n">
-        <v>874</v>
+        <v>887</v>
       </c>
       <c r="B127" t="n">
-        <v>0.3610796311341488</v>
+        <v>0.3217583741703381</v>
       </c>
       <c r="C127" t="n">
-        <v>0.238954363544711</v>
+        <v>0.3209856327912293</v>
       </c>
     </row>
     <row r="128">
       <c r="A128" t="n">
-        <v>864</v>
+        <v>876</v>
       </c>
       <c r="B128" t="n">
-        <v>0.3032921994982787</v>
+        <v>0.3490808065648447</v>
       </c>
       <c r="C128" t="n">
-        <v>0.1488743077229255</v>
+        <v>0.1408378652040445</v>
       </c>
     </row>
     <row r="129">
       <c r="A129" t="n">
-        <v>863</v>
+        <v>874</v>
       </c>
       <c r="B129" t="n">
-        <v>0.3256974475820567</v>
+        <v>0.3610796311341488</v>
       </c>
       <c r="C129" t="n">
-        <v>0.1879425499591285</v>
+        <v>0.238954363544711</v>
       </c>
     </row>
     <row r="130">
       <c r="A130" t="n">
-        <v>862</v>
+        <v>864</v>
       </c>
       <c r="B130" t="n">
-        <v>0.5887604521763219</v>
+        <v>0.3032936621157706</v>
       </c>
       <c r="C130" t="n">
-        <v>0.2349389855258899</v>
+        <v>0.1489170629055099</v>
       </c>
     </row>
     <row r="131">
       <c r="A131" t="n">
-        <v>861</v>
+        <v>863</v>
       </c>
       <c r="B131" t="n">
-        <v>0.3167810529762386</v>
+        <v>0.3256974475820567</v>
       </c>
       <c r="C131" t="n">
-        <v>0.1921135570225264</v>
+        <v>0.1879425499591285</v>
       </c>
     </row>
     <row r="132">
       <c r="A132" t="n">
-        <v>733</v>
+        <v>862</v>
       </c>
       <c r="B132" t="n">
-        <v>0.343957426640445</v>
+        <v>0.5887604521763219</v>
       </c>
       <c r="C132" t="n">
-        <v>0.2946109943963943</v>
+        <v>0.2349389855258899</v>
       </c>
     </row>
     <row r="133">
       <c r="A133" t="n">
-        <v>728</v>
+        <v>861</v>
       </c>
       <c r="B133" t="n">
-        <v>0.3452912417166399</v>
+        <v>0.3167810529762386</v>
       </c>
       <c r="C133" t="n">
-        <v>0.2813944014617442</v>
+        <v>0.1921135570225264</v>
       </c>
     </row>
     <row r="134">
       <c r="A134" t="n">
-        <v>727</v>
+        <v>733</v>
       </c>
       <c r="B134" t="n">
-        <v>0.3493932630422841</v>
+        <v>0.343957426640445</v>
       </c>
       <c r="C134" t="n">
-        <v>0.2340505526158381</v>
+        <v>0.2946109943963943</v>
       </c>
     </row>
     <row r="135">
       <c r="A135" t="n">
-        <v>710</v>
+        <v>728</v>
       </c>
       <c r="B135" t="n">
-        <v>0.3920208048396226</v>
+        <v>0.3452912417166399</v>
       </c>
       <c r="C135" t="n">
-        <v>0.3084731658007794</v>
+        <v>0.2813944014617442</v>
       </c>
     </row>
     <row r="136">
       <c r="A136" t="n">
-        <v>709</v>
+        <v>727</v>
       </c>
       <c r="B136" t="n">
-        <v>0.3770303255745312</v>
+        <v>0.3493932630422841</v>
       </c>
       <c r="C136" t="n">
-        <v>0.417394023590101</v>
+        <v>0.2340505526158381</v>
       </c>
     </row>
     <row r="137">
       <c r="A137" t="n">
-        <v>708</v>
+        <v>710</v>
       </c>
       <c r="B137" t="n">
-        <v>0.3532671931796519</v>
+        <v>0.3920208048396226</v>
       </c>
       <c r="C137" t="n">
-        <v>0.2801051729978689</v>
+        <v>0.3084731658007794</v>
       </c>
     </row>
     <row r="138">
       <c r="A138" t="n">
-        <v>703</v>
+        <v>709</v>
       </c>
       <c r="B138" t="n">
-        <v>0.3692771382504424</v>
+        <v>0.3770303255745312</v>
       </c>
       <c r="C138" t="n">
-        <v>0.2522378242698015</v>
+        <v>0.417394023590101</v>
       </c>
     </row>
     <row r="139">
       <c r="A139" t="n">
-        <v>699</v>
+        <v>708</v>
       </c>
       <c r="B139" t="n">
-        <v>0.4209821611508353</v>
+        <v>0.3532671931796519</v>
       </c>
       <c r="C139" t="n">
-        <v>0.2431552076022918</v>
+        <v>0.2801051729978689</v>
       </c>
     </row>
     <row r="140">
       <c r="A140" t="n">
-        <v>645</v>
+        <v>703</v>
       </c>
       <c r="B140" t="n">
-        <v>0.3350241609741931</v>
+        <v>0.3692435881529905</v>
       </c>
       <c r="C140" t="n">
-        <v>0.2930353422789901</v>
+        <v>0.2522407233200708</v>
       </c>
     </row>
     <row r="141">
       <c r="A141" t="n">
-        <v>642</v>
+        <v>699</v>
       </c>
       <c r="B141" t="n">
-        <v>0.2647797501931667</v>
+        <v>0.4209821611508353</v>
       </c>
       <c r="C141" t="n">
-        <v>0.1664603001366493</v>
+        <v>0.2431552076022918</v>
       </c>
     </row>
     <row r="142">
       <c r="A142" t="n">
-        <v>641</v>
+        <v>645</v>
       </c>
       <c r="B142" t="n">
-        <v>0.3958268962092519</v>
+        <v>0.3350241609741931</v>
       </c>
       <c r="C142" t="n">
-        <v>0.3236362580725322</v>
+        <v>0.2930353422789901</v>
       </c>
     </row>
     <row r="143">
       <c r="A143" t="n">
-        <v>47</v>
+        <v>642</v>
       </c>
       <c r="B143" t="n">
-        <v>0.3519491089564129</v>
+        <v>0.2647797501931667</v>
       </c>
       <c r="C143" t="n">
-        <v>0.3319633994983702</v>
+        <v>0.1664603001366493</v>
       </c>
     </row>
     <row r="144">
       <c r="A144" t="n">
-        <v>26</v>
+        <v>641</v>
       </c>
       <c r="B144" t="n">
-        <v>0.3505273733544978</v>
+        <v>0.3958268962092519</v>
       </c>
       <c r="C144" t="n">
-        <v>0.2801632709223243</v>
+        <v>0.3236362580725322</v>
       </c>
     </row>
     <row r="145">
       <c r="A145" t="n">
+        <v>47</v>
+      </c>
+      <c r="B145" t="n">
+        <v>0.3519491089564129</v>
+      </c>
+      <c r="C145" t="n">
+        <v>0.3319633994983702</v>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" t="n">
+        <v>26</v>
+      </c>
+      <c r="B146" t="n">
+        <v>0.3505273733544978</v>
+      </c>
+      <c r="C146" t="n">
+        <v>0.2801632709223243</v>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" t="n">
         <v>7</v>
       </c>
-      <c r="B145" t="n">
+      <c r="B147" t="n">
         <v>0.2758229919721963</v>
       </c>
-      <c r="C145" t="n">
+      <c r="C147" t="n">
         <v>0.1188680437542776</v>
       </c>
     </row>

</xml_diff>

<commit_message>
update on the hourly data
</commit_message>
<xml_diff>
--- a/hourly datasets/PlantID_year-4final.xlsx
+++ b/hourly datasets/PlantID_year-4final.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C147"/>
+  <dimension ref="A1:F147"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -441,7 +441,22 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
+          <t>CoefCat</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
           <t>intercept</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>cat_value_current</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>efficiencyMax</t>
         </is>
       </c>
     </row>
@@ -450,10 +465,21 @@
         <v>8226</v>
       </c>
       <c r="B2" t="n">
-        <v>0.3538135330166676</v>
-      </c>
-      <c r="C2" t="n">
+        <v>0.3549054033078188</v>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>105%&gt;gen/cap&gt;100%</t>
+        </is>
+      </c>
+      <c r="D2" t="n">
         <v>0.1546329437273875</v>
+      </c>
+      <c r="E2" t="n">
+        <v>0.2915500913161409</v>
+      </c>
+      <c r="F2" t="n">
+        <v>0.3813251109835441</v>
       </c>
     </row>
     <row r="3">
@@ -461,10 +487,21 @@
         <v>8102</v>
       </c>
       <c r="B3" t="n">
-        <v>0.3418311770192904</v>
-      </c>
-      <c r="C3" t="n">
+        <v>0.3447854962069838</v>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>110%&gt;gen/cap&gt;105%</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
         <v>0.2093754658246962</v>
+      </c>
+      <c r="E3" t="n">
+        <v>0.3429164079648739</v>
+      </c>
+      <c r="F3" t="n">
+        <v>0.3198388872339761</v>
       </c>
     </row>
     <row r="4">
@@ -474,8 +511,19 @@
       <c r="B4" t="n">
         <v>0.2831109832446886</v>
       </c>
-      <c r="C4" t="n">
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>55%&gt;gen/cap&gt;50%</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
         <v>0.2596568808986405</v>
+      </c>
+      <c r="E4" t="n">
+        <v>0.3299146687852249</v>
+      </c>
+      <c r="F4" t="n">
+        <v>0.2711661134513298</v>
       </c>
     </row>
     <row r="5">
@@ -485,8 +533,19 @@
       <c r="B5" t="n">
         <v>0.2861244128230339</v>
       </c>
-      <c r="C5" t="n">
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>50%&gt;gen/cap&gt;45%</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
         <v>0.2117030783728674</v>
+      </c>
+      <c r="E5" t="n">
+        <v>0.3290786474885763</v>
+      </c>
+      <c r="F5" t="n">
+        <v>0.2750155643263237</v>
       </c>
     </row>
     <row r="6">
@@ -496,8 +555,19 @@
       <c r="B6" t="n">
         <v>0.2811489327152589</v>
       </c>
-      <c r="C6" t="n">
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>85%&gt;gen/cap&gt;80%</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
         <v>0.1373650061817846</v>
+      </c>
+      <c r="E6" t="n">
+        <v>0.327678763896358</v>
+      </c>
+      <c r="F6" t="n">
+        <v>0.2714399678107671</v>
       </c>
     </row>
     <row r="7">
@@ -505,10 +575,21 @@
         <v>6705</v>
       </c>
       <c r="B7" t="n">
-        <v>0.3027577199662704</v>
-      </c>
-      <c r="C7" t="n">
+        <v>0.3662226043901747</v>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>120%&gt;gen/cap&gt;115%</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
         <v>0.07713924339506242</v>
+      </c>
+      <c r="E7" t="n">
+        <v>0.3715206539768175</v>
+      </c>
+      <c r="F7" t="n">
+        <v>0.3126717494052234</v>
       </c>
     </row>
     <row r="8">
@@ -518,8 +599,19 @@
       <c r="B8" t="n">
         <v>0.3241001533599427</v>
       </c>
-      <c r="C8" t="n">
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>85%&gt;gen/cap&gt;80%</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
         <v>0.1687395391009784</v>
+      </c>
+      <c r="E8" t="n">
+        <v>0.327678763896358</v>
+      </c>
+      <c r="F8" t="n">
+        <v>0.3143911884554509</v>
       </c>
     </row>
     <row r="9">
@@ -527,10 +619,21 @@
         <v>6195</v>
       </c>
       <c r="B9" t="n">
-        <v>1.13589443031268</v>
-      </c>
-      <c r="C9" t="n">
+        <v>0.5141986897576902</v>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>60%&gt;gen/cap&gt;55%</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
         <v>0.1922063364081459</v>
+      </c>
+      <c r="E9" t="n">
+        <v>0.3300662278897786</v>
+      </c>
+      <c r="F9" t="n">
+        <v>0.5021022608597778</v>
       </c>
     </row>
     <row r="10">
@@ -540,8 +643,19 @@
       <c r="B10" t="n">
         <v>0.372197564978325</v>
       </c>
-      <c r="C10" t="n">
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>20%&gt;gen/cap&gt;15%</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
         <v>0.2390211436427051</v>
+      </c>
+      <c r="E10" t="n">
+        <v>0.3027123616367527</v>
+      </c>
+      <c r="F10" t="n">
+        <v>0.3874550023334385</v>
       </c>
     </row>
     <row r="11">
@@ -549,10 +663,21 @@
         <v>6124</v>
       </c>
       <c r="B11" t="n">
-        <v>0.4459275072059499</v>
-      </c>
-      <c r="C11" t="n">
+        <v>0.3595520120231962</v>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>25%&gt;gen/cap&gt;20%</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
         <v>0.3260796095772839</v>
+      </c>
+      <c r="E11" t="n">
+        <v>0.3119528493677421</v>
+      </c>
+      <c r="F11" t="n">
+        <v>0.3655689616473203</v>
       </c>
     </row>
     <row r="12">
@@ -562,8 +687,19 @@
       <c r="B12" t="n">
         <v>0.4221246486283537</v>
       </c>
-      <c r="C12" t="n">
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>65%&gt;gen/cap&gt;60%</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
         <v>0.2749164335955042</v>
+      </c>
+      <c r="E12" t="n">
+        <v>0.3252929965811113</v>
+      </c>
+      <c r="F12" t="n">
+        <v>0.4148014510391086</v>
       </c>
     </row>
     <row r="13">
@@ -573,8 +709,19 @@
       <c r="B13" t="n">
         <v>0.2797165207697392</v>
       </c>
-      <c r="C13" t="n">
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>90%&gt;gen/cap&gt;85%</t>
+        </is>
+      </c>
+      <c r="D13" t="n">
         <v>0.1400301505202271</v>
+      </c>
+      <c r="E13" t="n">
+        <v>0.3261577166574556</v>
+      </c>
+      <c r="F13" t="n">
+        <v>0.2715286031041498</v>
       </c>
     </row>
     <row r="14">
@@ -584,8 +731,19 @@
       <c r="B14" t="n">
         <v>0.3860563094385062</v>
       </c>
-      <c r="C14" t="n">
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>60%&gt;gen/cap&gt;55%</t>
+        </is>
+      </c>
+      <c r="D14" t="n">
         <v>0.284698748832014</v>
+      </c>
+      <c r="E14" t="n">
+        <v>0.3300662278897786</v>
+      </c>
+      <c r="F14" t="n">
+        <v>0.3739598805405938</v>
       </c>
     </row>
     <row r="15">
@@ -595,8 +753,19 @@
       <c r="B15" t="n">
         <v>0.3540131886687025</v>
       </c>
-      <c r="C15" t="n">
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>15%&gt;gen/cap&gt;10%</t>
+        </is>
+      </c>
+      <c r="D15" t="n">
         <v>0.3175453004912062</v>
+      </c>
+      <c r="E15" t="n">
+        <v>0.2861617054590648</v>
+      </c>
+      <c r="F15" t="n">
+        <v>0.3858212822015039</v>
       </c>
     </row>
     <row r="16">
@@ -606,8 +775,19 @@
       <c r="B16" t="n">
         <v>0.3265982377456648</v>
       </c>
-      <c r="C16" t="n">
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>45%&gt;gen/cap&gt;40%</t>
+        </is>
+      </c>
+      <c r="D16" t="n">
         <v>0.2158015486361115</v>
+      </c>
+      <c r="E16" t="n">
+        <v>0.3259006427158213</v>
+      </c>
+      <c r="F16" t="n">
+        <v>0.3186673940217097</v>
       </c>
     </row>
     <row r="17">
@@ -617,8 +797,19 @@
       <c r="B17" t="n">
         <v>0.2997548580286813</v>
       </c>
-      <c r="C17" t="n">
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>50%&gt;gen/cap&gt;45%</t>
+        </is>
+      </c>
+      <c r="D17" t="n">
         <v>0.2939386487086316</v>
+      </c>
+      <c r="E17" t="n">
+        <v>0.3290786474885763</v>
+      </c>
+      <c r="F17" t="n">
+        <v>0.2886460095319711</v>
       </c>
     </row>
     <row r="18">
@@ -628,8 +819,19 @@
       <c r="B18" t="n">
         <v>0.3826035625465314</v>
       </c>
-      <c r="C18" t="n">
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>30%&gt;gen/cap&gt;25%</t>
+        </is>
+      </c>
+      <c r="D18" t="n">
         <v>0.3574954265024484</v>
+      </c>
+      <c r="E18" t="n">
+        <v>0.317495714201756</v>
+      </c>
+      <c r="F18" t="n">
+        <v>0.3830776473366416</v>
       </c>
     </row>
     <row r="19">
@@ -637,10 +839,21 @@
         <v>6041</v>
       </c>
       <c r="B19" t="n">
-        <v>0.3616478261929838</v>
-      </c>
-      <c r="C19" t="n">
+        <v>0.3517464985360521</v>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>30%&gt;gen/cap&gt;25%</t>
+        </is>
+      </c>
+      <c r="D19" t="n">
         <v>0.2740011414567843</v>
+      </c>
+      <c r="E19" t="n">
+        <v>0.317495714201756</v>
+      </c>
+      <c r="F19" t="n">
+        <v>0.3522205833261623</v>
       </c>
     </row>
     <row r="20">
@@ -648,10 +861,21 @@
         <v>6025</v>
       </c>
       <c r="B20" t="n">
-        <v>0.3965486879255518</v>
-      </c>
-      <c r="C20" t="n">
+        <v>0.4044542204277208</v>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>105%&gt;gen/cap&gt;100%</t>
+        </is>
+      </c>
+      <c r="D20" t="n">
         <v>0.1934815315117472</v>
+      </c>
+      <c r="E20" t="n">
+        <v>0.2915500913161409</v>
+      </c>
+      <c r="F20" t="n">
+        <v>0.4308739281034461</v>
       </c>
     </row>
     <row r="21">
@@ -659,10 +883,21 @@
         <v>6018</v>
       </c>
       <c r="B21" t="n">
-        <v>0.3359241691763017</v>
-      </c>
-      <c r="C21" t="n">
+        <v>0.3471524897114325</v>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>105%&gt;gen/cap&gt;100%</t>
+        </is>
+      </c>
+      <c r="D21" t="n">
         <v>0.2038559471964597</v>
+      </c>
+      <c r="E21" t="n">
+        <v>0.2915500913161409</v>
+      </c>
+      <c r="F21" t="n">
+        <v>0.3735721973871578</v>
       </c>
     </row>
     <row r="22">
@@ -672,8 +907,19 @@
       <c r="B22" t="n">
         <v>0.3642751313647442</v>
       </c>
-      <c r="C22" t="n">
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>100%&gt;gen/cap&gt;95%</t>
+        </is>
+      </c>
+      <c r="D22" t="n">
         <v>0.1796301357976015</v>
+      </c>
+      <c r="E22" t="n">
+        <v>0.3179697989918662</v>
+      </c>
+      <c r="F22" t="n">
+        <v>0.3642751313647441</v>
       </c>
     </row>
     <row r="23">
@@ -683,8 +929,19 @@
       <c r="B23" t="n">
         <v>0.2878529632520799</v>
       </c>
-      <c r="C23" t="n">
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>80%&gt;gen/cap&gt;75%</t>
+        </is>
+      </c>
+      <c r="D23" t="n">
         <v>0.1641334652606165</v>
+      </c>
+      <c r="E23" t="n">
+        <v>0.3260855209567263</v>
+      </c>
+      <c r="F23" t="n">
+        <v>0.2797372412872198</v>
       </c>
     </row>
     <row r="24">
@@ -692,10 +949,21 @@
         <v>4078</v>
       </c>
       <c r="B24" t="n">
-        <v>0.3347993193356881</v>
-      </c>
-      <c r="C24" t="n">
+        <v>0.2984798514966398</v>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>15%&gt;gen/cap&gt;10%</t>
+        </is>
+      </c>
+      <c r="D24" t="n">
         <v>0.2746844040044751</v>
+      </c>
+      <c r="E24" t="n">
+        <v>0.2861617054590648</v>
+      </c>
+      <c r="F24" t="n">
+        <v>0.3302879450294412</v>
       </c>
     </row>
     <row r="25">
@@ -705,8 +973,19 @@
       <c r="B25" t="n">
         <v>0.3102934197759805</v>
       </c>
-      <c r="C25" t="n">
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>55%&gt;gen/cap&gt;50%</t>
+        </is>
+      </c>
+      <c r="D25" t="n">
         <v>0.2821073164834376</v>
+      </c>
+      <c r="E25" t="n">
+        <v>0.3299146687852249</v>
+      </c>
+      <c r="F25" t="n">
+        <v>0.2983485499826218</v>
       </c>
     </row>
     <row r="26">
@@ -714,10 +993,21 @@
         <v>4057</v>
       </c>
       <c r="B26" t="n">
-        <v>0.3569403101835894</v>
-      </c>
-      <c r="C26" t="n">
+        <v>0.3027102758833422</v>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>35%&gt;gen/cap&gt;30%</t>
+        </is>
+      </c>
+      <c r="D26" t="n">
         <v>0.2832344266904956</v>
+      </c>
+      <c r="E26" t="n">
+        <v>0.3228360886967814</v>
+      </c>
+      <c r="F26" t="n">
+        <v>0.2978439861784269</v>
       </c>
     </row>
     <row r="27">
@@ -725,10 +1015,21 @@
         <v>4054</v>
       </c>
       <c r="B27" t="n">
-        <v>0.3699932106602539</v>
-      </c>
-      <c r="C27" t="n">
+        <v>0.4109031674659835</v>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>120%&gt;gen/cap&gt;115%</t>
+        </is>
+      </c>
+      <c r="D27" t="n">
         <v>0.2259581061908454</v>
+      </c>
+      <c r="E27" t="n">
+        <v>0.3715206539768175</v>
+      </c>
+      <c r="F27" t="n">
+        <v>0.3573523124810322</v>
       </c>
     </row>
     <row r="28">
@@ -738,8 +1039,19 @@
       <c r="B28" t="n">
         <v>0.3533299368859437</v>
       </c>
-      <c r="C28" t="n">
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>40%&gt;gen/cap&gt;35%</t>
+        </is>
+      </c>
+      <c r="D28" t="n">
         <v>0.3641465745337381</v>
+      </c>
+      <c r="E28" t="n">
+        <v>0.3252845350267428</v>
+      </c>
+      <c r="F28" t="n">
+        <v>0.3460152008510671</v>
       </c>
     </row>
     <row r="29">
@@ -749,8 +1061,19 @@
       <c r="B29" t="n">
         <v>0.3590737138840505</v>
       </c>
-      <c r="C29" t="n">
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>100%&gt;gen/cap&gt;95%</t>
+        </is>
+      </c>
+      <c r="D29" t="n">
         <v>0.2126324603695098</v>
+      </c>
+      <c r="E29" t="n">
+        <v>0.3179697989918662</v>
+      </c>
+      <c r="F29" t="n">
+        <v>0.3590737138840505</v>
       </c>
     </row>
     <row r="30">
@@ -760,8 +1083,19 @@
       <c r="B30" t="n">
         <v>0.2846702677350387</v>
       </c>
-      <c r="C30" t="n">
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>60%&gt;gen/cap&gt;55%</t>
+        </is>
+      </c>
+      <c r="D30" t="n">
         <v>0.2356623440553718</v>
+      </c>
+      <c r="E30" t="n">
+        <v>0.3300662278897786</v>
+      </c>
+      <c r="F30" t="n">
+        <v>0.2725738388371264</v>
       </c>
     </row>
     <row r="31">
@@ -771,8 +1105,19 @@
       <c r="B31" t="n">
         <v>0.3628827346266098</v>
       </c>
-      <c r="C31" t="n">
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>95%&gt;gen/cap&gt;90%</t>
+        </is>
+      </c>
+      <c r="D31" t="n">
         <v>0.2133958277579524</v>
+      </c>
+      <c r="E31" t="n">
+        <v>0.3266645889845783</v>
+      </c>
+      <c r="F31" t="n">
+        <v>0.3541879446338977</v>
       </c>
     </row>
     <row r="32">
@@ -782,8 +1127,19 @@
       <c r="B32" t="n">
         <v>0.3719535146340285</v>
       </c>
-      <c r="C32" t="n">
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>35%&gt;gen/cap&gt;30%</t>
+        </is>
+      </c>
+      <c r="D32" t="n">
         <v>0.2492150820300328</v>
+      </c>
+      <c r="E32" t="n">
+        <v>0.3228360886967814</v>
+      </c>
+      <c r="F32" t="n">
+        <v>0.3670872249291132</v>
       </c>
     </row>
     <row r="33">
@@ -793,8 +1149,19 @@
       <c r="B33" t="n">
         <v>0.3974771691341019</v>
       </c>
-      <c r="C33" t="n">
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>35%&gt;gen/cap&gt;30%</t>
+        </is>
+      </c>
+      <c r="D33" t="n">
         <v>0.3791859625391745</v>
+      </c>
+      <c r="E33" t="n">
+        <v>0.3228360886967814</v>
+      </c>
+      <c r="F33" t="n">
+        <v>0.3926108794291867</v>
       </c>
     </row>
     <row r="34">
@@ -804,8 +1171,19 @@
       <c r="B34" t="n">
         <v>0.3655394713647989</v>
       </c>
-      <c r="C34" t="n">
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>35%&gt;gen/cap&gt;30%</t>
+        </is>
+      </c>
+      <c r="D34" t="n">
         <v>0.1685614844142961</v>
+      </c>
+      <c r="E34" t="n">
+        <v>0.3228360886967814</v>
+      </c>
+      <c r="F34" t="n">
+        <v>0.3606731816598837</v>
       </c>
     </row>
     <row r="35">
@@ -815,8 +1193,19 @@
       <c r="B35" t="n">
         <v>0.2981242612393976</v>
       </c>
-      <c r="C35" t="n">
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>35%&gt;gen/cap&gt;30%</t>
+        </is>
+      </c>
+      <c r="D35" t="n">
         <v>0.1924259713607003</v>
+      </c>
+      <c r="E35" t="n">
+        <v>0.3228360886967814</v>
+      </c>
+      <c r="F35" t="n">
+        <v>0.2932579715344822</v>
       </c>
     </row>
     <row r="36">
@@ -826,8 +1215,19 @@
       <c r="B36" t="n">
         <v>0.3648328457447845</v>
       </c>
-      <c r="C36" t="n">
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>20%&gt;gen/cap&gt;15%</t>
+        </is>
+      </c>
+      <c r="D36" t="n">
         <v>0.2581656114698205</v>
+      </c>
+      <c r="E36" t="n">
+        <v>0.3027123616367527</v>
+      </c>
+      <c r="F36" t="n">
+        <v>0.380090283099898</v>
       </c>
     </row>
     <row r="37">
@@ -837,8 +1237,19 @@
       <c r="B37" t="n">
         <v>0.3512559772993038</v>
       </c>
-      <c r="C37" t="n">
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>50%&gt;gen/cap&gt;45%</t>
+        </is>
+      </c>
+      <c r="D37" t="n">
         <v>0.2095801473789035</v>
+      </c>
+      <c r="E37" t="n">
+        <v>0.3290786474885763</v>
+      </c>
+      <c r="F37" t="n">
+        <v>0.3401471288025936</v>
       </c>
     </row>
     <row r="38">
@@ -848,8 +1259,19 @@
       <c r="B38" t="n">
         <v>0.3407233675796342</v>
       </c>
-      <c r="C38" t="n">
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>50%&gt;gen/cap&gt;45%</t>
+        </is>
+      </c>
+      <c r="D38" t="n">
         <v>0.2276726085644257</v>
+      </c>
+      <c r="E38" t="n">
+        <v>0.3290786474885763</v>
+      </c>
+      <c r="F38" t="n">
+        <v>0.329614519082924</v>
       </c>
     </row>
     <row r="39">
@@ -857,10 +1279,21 @@
         <v>3406</v>
       </c>
       <c r="B39" t="n">
-        <v>0.390122505563438</v>
-      </c>
-      <c r="C39" t="n">
+        <v>0.3589678315352208</v>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>55%&gt;gen/cap&gt;50%</t>
+        </is>
+      </c>
+      <c r="D39" t="n">
         <v>0.3361995570496853</v>
+      </c>
+      <c r="E39" t="n">
+        <v>0.3299146687852249</v>
+      </c>
+      <c r="F39" t="n">
+        <v>0.3470229617418621</v>
       </c>
     </row>
     <row r="40">
@@ -870,8 +1303,19 @@
       <c r="B40" t="n">
         <v>0.3750804470195317</v>
       </c>
-      <c r="C40" t="n">
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>40%&gt;gen/cap&gt;35%</t>
+        </is>
+      </c>
+      <c r="D40" t="n">
         <v>0.3403961674696739</v>
+      </c>
+      <c r="E40" t="n">
+        <v>0.3252845350267428</v>
+      </c>
+      <c r="F40" t="n">
+        <v>0.367765710984655</v>
       </c>
     </row>
     <row r="41">
@@ -881,8 +1325,19 @@
       <c r="B41" t="n">
         <v>0.3027905338467628</v>
       </c>
-      <c r="C41" t="n">
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>55%&gt;gen/cap&gt;50%</t>
+        </is>
+      </c>
+      <c r="D41" t="n">
         <v>0.1372195411025252</v>
+      </c>
+      <c r="E41" t="n">
+        <v>0.3299146687852249</v>
+      </c>
+      <c r="F41" t="n">
+        <v>0.2908456640534041</v>
       </c>
     </row>
     <row r="42">
@@ -892,8 +1347,19 @@
       <c r="B42" t="n">
         <v>0.4532756263660066</v>
       </c>
-      <c r="C42" t="n">
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>30%&gt;gen/cap&gt;25%</t>
+        </is>
+      </c>
+      <c r="D42" t="n">
         <v>0.4428329400054485</v>
+      </c>
+      <c r="E42" t="n">
+        <v>0.317495714201756</v>
+      </c>
+      <c r="F42" t="n">
+        <v>0.4537497111561168</v>
       </c>
     </row>
     <row r="43">
@@ -903,8 +1369,19 @@
       <c r="B43" t="n">
         <v>0.3283487846149303</v>
       </c>
-      <c r="C43" t="n">
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>60%&gt;gen/cap&gt;55%</t>
+        </is>
+      </c>
+      <c r="D43" t="n">
         <v>0.1800673204823876</v>
+      </c>
+      <c r="E43" t="n">
+        <v>0.3300662278897786</v>
+      </c>
+      <c r="F43" t="n">
+        <v>0.3162523557170179</v>
       </c>
     </row>
     <row r="44">
@@ -914,8 +1391,19 @@
       <c r="B44" t="n">
         <v>0.3697419581629559</v>
       </c>
-      <c r="C44" t="n">
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>100%&gt;gen/cap&gt;95%</t>
+        </is>
+      </c>
+      <c r="D44" t="n">
         <v>0.2357506535012228</v>
+      </c>
+      <c r="E44" t="n">
+        <v>0.3179697989918662</v>
+      </c>
+      <c r="F44" t="n">
+        <v>0.3697419581629559</v>
       </c>
     </row>
     <row r="45">
@@ -925,8 +1413,19 @@
       <c r="B45" t="n">
         <v>0.3373794246937235</v>
       </c>
-      <c r="C45" t="n">
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>90%&gt;gen/cap&gt;85%</t>
+        </is>
+      </c>
+      <c r="D45" t="n">
         <v>0.1771704758366996</v>
+      </c>
+      <c r="E45" t="n">
+        <v>0.3261577166574556</v>
+      </c>
+      <c r="F45" t="n">
+        <v>0.3291915070281341</v>
       </c>
     </row>
     <row r="46">
@@ -936,8 +1435,19 @@
       <c r="B46" t="n">
         <v>0.56709112999304</v>
       </c>
-      <c r="C46" t="n">
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>95%&gt;gen/cap&gt;90%</t>
+        </is>
+      </c>
+      <c r="D46" t="n">
         <v>0.4966341528697863</v>
+      </c>
+      <c r="E46" t="n">
+        <v>0.3266645889845783</v>
+      </c>
+      <c r="F46" t="n">
+        <v>0.5583963400003279</v>
       </c>
     </row>
     <row r="47">
@@ -947,8 +1457,19 @@
       <c r="B47" t="n">
         <v>0.3223629328616754</v>
       </c>
-      <c r="C47" t="n">
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>95%&gt;gen/cap&gt;90%</t>
+        </is>
+      </c>
+      <c r="D47" t="n">
         <v>0.2891267738276887</v>
+      </c>
+      <c r="E47" t="n">
+        <v>0.3266645889845783</v>
+      </c>
+      <c r="F47" t="n">
+        <v>0.3136681428689634</v>
       </c>
     </row>
     <row r="48">
@@ -958,8 +1479,19 @@
       <c r="B48" t="n">
         <v>0.3608692261421088</v>
       </c>
-      <c r="C48" t="n">
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>90%&gt;gen/cap&gt;85%</t>
+        </is>
+      </c>
+      <c r="D48" t="n">
         <v>0.3227148099598149</v>
+      </c>
+      <c r="E48" t="n">
+        <v>0.3261577166574556</v>
+      </c>
+      <c r="F48" t="n">
+        <v>0.3526813084765194</v>
       </c>
     </row>
     <row r="49">
@@ -969,8 +1501,19 @@
       <c r="B49" t="n">
         <v>0.3560229317470405</v>
       </c>
-      <c r="C49" t="n">
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>100%&gt;gen/cap&gt;95%</t>
+        </is>
+      </c>
+      <c r="D49" t="n">
         <v>0.3031239627150191</v>
+      </c>
+      <c r="E49" t="n">
+        <v>0.3179697989918662</v>
+      </c>
+      <c r="F49" t="n">
+        <v>0.3560229317470405</v>
       </c>
     </row>
     <row r="50">
@@ -980,8 +1523,19 @@
       <c r="B50" t="n">
         <v>0.3644217095493537</v>
       </c>
-      <c r="C50" t="n">
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>30%&gt;gen/cap&gt;25%</t>
+        </is>
+      </c>
+      <c r="D50" t="n">
         <v>0.3072503879074647</v>
+      </c>
+      <c r="E50" t="n">
+        <v>0.317495714201756</v>
+      </c>
+      <c r="F50" t="n">
+        <v>0.3648957943394638</v>
       </c>
     </row>
     <row r="51">
@@ -991,8 +1545,19 @@
       <c r="B51" t="n">
         <v>0.3870997564043199</v>
       </c>
-      <c r="C51" t="n">
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>95%&gt;gen/cap&gt;90%</t>
+        </is>
+      </c>
+      <c r="D51" t="n">
         <v>0.1611534039363451</v>
+      </c>
+      <c r="E51" t="n">
+        <v>0.3266645889845783</v>
+      </c>
+      <c r="F51" t="n">
+        <v>0.3784049664116078</v>
       </c>
     </row>
     <row r="52">
@@ -1000,10 +1565,21 @@
         <v>2878</v>
       </c>
       <c r="B52" t="n">
-        <v>0.3731426453658845</v>
-      </c>
-      <c r="C52" t="n">
+        <v>0.3771958640730231</v>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>105%&gt;gen/cap&gt;100%</t>
+        </is>
+      </c>
+      <c r="D52" t="n">
         <v>0.3766221542515145</v>
+      </c>
+      <c r="E52" t="n">
+        <v>0.2915500913161409</v>
+      </c>
+      <c r="F52" t="n">
+        <v>0.4036155717487483</v>
       </c>
     </row>
     <row r="53">
@@ -1011,10 +1587,21 @@
         <v>2876</v>
       </c>
       <c r="B53" t="n">
-        <v>0.3714344482390222</v>
-      </c>
-      <c r="C53" t="n">
+        <v>0.3934318819363984</v>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>110%&gt;gen/cap&gt;105%</t>
+        </is>
+      </c>
+      <c r="D53" t="n">
         <v>0.3753520536981952</v>
+      </c>
+      <c r="E53" t="n">
+        <v>0.3429164079648739</v>
+      </c>
+      <c r="F53" t="n">
+        <v>0.3684852729633907</v>
       </c>
     </row>
     <row r="54">
@@ -1024,8 +1611,19 @@
       <c r="B54" t="n">
         <v>0.3816908723548493</v>
       </c>
-      <c r="C54" t="n">
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>95%&gt;gen/cap&gt;90%</t>
+        </is>
+      </c>
+      <c r="D54" t="n">
         <v>0.3822033877803676</v>
+      </c>
+      <c r="E54" t="n">
+        <v>0.3266645889845783</v>
+      </c>
+      <c r="F54" t="n">
+        <v>0.3729960823621372</v>
       </c>
     </row>
     <row r="55">
@@ -1033,10 +1631,21 @@
         <v>2866</v>
       </c>
       <c r="B55" t="n">
-        <v>0.3485492409531383</v>
-      </c>
-      <c r="C55" t="n">
+        <v>0.3411841968867677</v>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>50%&gt;gen/cap&gt;45%</t>
+        </is>
+      </c>
+      <c r="D55" t="n">
         <v>0.2695872999860202</v>
+      </c>
+      <c r="E55" t="n">
+        <v>0.3290786474885763</v>
+      </c>
+      <c r="F55" t="n">
+        <v>0.3300753483900575</v>
       </c>
     </row>
     <row r="56">
@@ -1046,8 +1655,19 @@
       <c r="B56" t="n">
         <v>0.3412229408875688</v>
       </c>
-      <c r="C56" t="n">
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>45%&gt;gen/cap&gt;40%</t>
+        </is>
+      </c>
+      <c r="D56" t="n">
         <v>0.2364963427400908</v>
+      </c>
+      <c r="E56" t="n">
+        <v>0.3259006427158213</v>
+      </c>
+      <c r="F56" t="n">
+        <v>0.3332920971636137</v>
       </c>
     </row>
     <row r="57">
@@ -1055,10 +1675,21 @@
         <v>2857</v>
       </c>
       <c r="B57" t="n">
-        <v>0.3824294957911895</v>
-      </c>
-      <c r="C57" t="n">
+        <v>0.3283616219426073</v>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>25%&gt;gen/cap&gt;20%</t>
+        </is>
+      </c>
+      <c r="D57" t="n">
         <v>0.2678828051140654</v>
+      </c>
+      <c r="E57" t="n">
+        <v>0.3119528493677421</v>
+      </c>
+      <c r="F57" t="n">
+        <v>0.3343785715667314</v>
       </c>
     </row>
     <row r="58">
@@ -1068,8 +1699,19 @@
       <c r="B58" t="n">
         <v>0.3579566481111134</v>
       </c>
-      <c r="C58" t="n">
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>75%&gt;gen/cap&gt;70%</t>
+        </is>
+      </c>
+      <c r="D58" t="n">
         <v>0.3558764325899996</v>
+      </c>
+      <c r="E58" t="n">
+        <v>0.3255475458727413</v>
+      </c>
+      <c r="F58" t="n">
+        <v>0.3503789012302383</v>
       </c>
     </row>
     <row r="59">
@@ -1079,8 +1721,19 @@
       <c r="B59" t="n">
         <v>0.3135601166183295</v>
       </c>
-      <c r="C59" t="n">
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>35%&gt;gen/cap&gt;30%</t>
+        </is>
+      </c>
+      <c r="D59" t="n">
         <v>0.1829303134549639</v>
+      </c>
+      <c r="E59" t="n">
+        <v>0.3228360886967814</v>
+      </c>
+      <c r="F59" t="n">
+        <v>0.3086938269134142</v>
       </c>
     </row>
     <row r="60">
@@ -1090,8 +1743,19 @@
       <c r="B60" t="n">
         <v>0.3621813144046631</v>
       </c>
-      <c r="C60" t="n">
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>55%&gt;gen/cap&gt;50%</t>
+        </is>
+      </c>
+      <c r="D60" t="n">
         <v>0.3094982158190912</v>
+      </c>
+      <c r="E60" t="n">
+        <v>0.3299146687852249</v>
+      </c>
+      <c r="F60" t="n">
+        <v>0.3502364446113044</v>
       </c>
     </row>
     <row r="61">
@@ -1099,10 +1763,21 @@
         <v>2838</v>
       </c>
       <c r="B61" t="n">
-        <v>2.604304879396142</v>
-      </c>
-      <c r="C61" t="n">
+        <v>0.434553870013095</v>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>40%&gt;gen/cap&gt;35%</t>
+        </is>
+      </c>
+      <c r="D61" t="n">
         <v>0.08878850733104968</v>
+      </c>
+      <c r="E61" t="n">
+        <v>0.3252845350267428</v>
+      </c>
+      <c r="F61" t="n">
+        <v>0.4272391339782183</v>
       </c>
     </row>
     <row r="62">
@@ -1112,8 +1787,19 @@
       <c r="B62" t="n">
         <v>0.3791077949882992</v>
       </c>
-      <c r="C62" t="n">
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>80%&gt;gen/cap&gt;75%</t>
+        </is>
+      </c>
+      <c r="D62" t="n">
         <v>0.2795475628018562</v>
+      </c>
+      <c r="E62" t="n">
+        <v>0.3260855209567263</v>
+      </c>
+      <c r="F62" t="n">
+        <v>0.3709920730234391</v>
       </c>
     </row>
     <row r="63">
@@ -1123,8 +1809,19 @@
       <c r="B63" t="n">
         <v>0.3497206129677597</v>
       </c>
-      <c r="C63" t="n">
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>25%&gt;gen/cap&gt;20%</t>
+        </is>
+      </c>
+      <c r="D63" t="n">
         <v>0.1265192524180493</v>
+      </c>
+      <c r="E63" t="n">
+        <v>0.3119528493677421</v>
+      </c>
+      <c r="F63" t="n">
+        <v>0.3557375625918838</v>
       </c>
     </row>
     <row r="64">
@@ -1132,10 +1829,21 @@
         <v>2835</v>
       </c>
       <c r="B64" t="n">
-        <v>0.4834529714480031</v>
-      </c>
-      <c r="C64" t="n">
+        <v>0.3827841863093921</v>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>40%&gt;gen/cap&gt;35%</t>
+        </is>
+      </c>
+      <c r="D64" t="n">
         <v>0.3225488769773652</v>
+      </c>
+      <c r="E64" t="n">
+        <v>0.3252845350267428</v>
+      </c>
+      <c r="F64" t="n">
+        <v>0.3754694502745155</v>
       </c>
     </row>
     <row r="65">
@@ -1145,8 +1853,19 @@
       <c r="B65" t="n">
         <v>0.3332437817966996</v>
       </c>
-      <c r="C65" t="n">
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>30%&gt;gen/cap&gt;25%</t>
+        </is>
+      </c>
+      <c r="D65" t="n">
         <v>0.3207110353591079</v>
+      </c>
+      <c r="E65" t="n">
+        <v>0.317495714201756</v>
+      </c>
+      <c r="F65" t="n">
+        <v>0.3337178665868097</v>
       </c>
     </row>
     <row r="66">
@@ -1156,8 +1875,19 @@
       <c r="B66" t="n">
         <v>0.35594901205693</v>
       </c>
-      <c r="C66" t="n">
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>20%&gt;gen/cap&gt;15%</t>
+        </is>
+      </c>
+      <c r="D66" t="n">
         <v>0.3267552515939188</v>
+      </c>
+      <c r="E66" t="n">
+        <v>0.3027123616367527</v>
+      </c>
+      <c r="F66" t="n">
+        <v>0.3712064494120434</v>
       </c>
     </row>
     <row r="67">
@@ -1167,8 +1897,19 @@
       <c r="B67" t="n">
         <v>0.3579022467365578</v>
       </c>
-      <c r="C67" t="n">
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>55%&gt;gen/cap&gt;50%</t>
+        </is>
+      </c>
+      <c r="D67" t="n">
         <v>0.2415511146651811</v>
+      </c>
+      <c r="E67" t="n">
+        <v>0.3299146687852249</v>
+      </c>
+      <c r="F67" t="n">
+        <v>0.3459573769431991</v>
       </c>
     </row>
     <row r="68">
@@ -1176,10 +1917,21 @@
         <v>2594</v>
       </c>
       <c r="B68" t="n">
-        <v>0.3870171691183409</v>
-      </c>
-      <c r="C68" t="n">
+        <v>0.3023649521725463</v>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>40%&gt;gen/cap&gt;35%</t>
+        </is>
+      </c>
+      <c r="D68" t="n">
         <v>0.2421771107376635</v>
+      </c>
+      <c r="E68" t="n">
+        <v>0.3252845350267428</v>
+      </c>
+      <c r="F68" t="n">
+        <v>0.2950502161376696</v>
       </c>
     </row>
     <row r="69">
@@ -1189,8 +1941,19 @@
       <c r="B69" t="n">
         <v>0.4007194333090533</v>
       </c>
-      <c r="C69" t="n">
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>50%&gt;gen/cap&gt;45%</t>
+        </is>
+      </c>
+      <c r="D69" t="n">
         <v>0.3033797962161246</v>
+      </c>
+      <c r="E69" t="n">
+        <v>0.3290786474885763</v>
+      </c>
+      <c r="F69" t="n">
+        <v>0.3896105848123432</v>
       </c>
     </row>
     <row r="70">
@@ -1200,8 +1963,19 @@
       <c r="B70" t="n">
         <v>0.3190059885038629</v>
       </c>
-      <c r="C70" t="n">
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>75%&gt;gen/cap&gt;70%</t>
+        </is>
+      </c>
+      <c r="D70" t="n">
         <v>0.3150614873796498</v>
+      </c>
+      <c r="E70" t="n">
+        <v>0.3255475458727413</v>
+      </c>
+      <c r="F70" t="n">
+        <v>0.3114282416229878</v>
       </c>
     </row>
     <row r="71">
@@ -1211,8 +1985,19 @@
       <c r="B71" t="n">
         <v>0.3749280884543377</v>
       </c>
-      <c r="C71" t="n">
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>15%&gt;gen/cap&gt;10%</t>
+        </is>
+      </c>
+      <c r="D71" t="n">
         <v>0.2527244504894599</v>
+      </c>
+      <c r="E71" t="n">
+        <v>0.2861617054590648</v>
+      </c>
+      <c r="F71" t="n">
+        <v>0.4067361819871391</v>
       </c>
     </row>
     <row r="72">
@@ -1222,8 +2007,19 @@
       <c r="B72" t="n">
         <v>0.3698113610556444</v>
       </c>
-      <c r="C72" t="n">
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>80%&gt;gen/cap&gt;75%</t>
+        </is>
+      </c>
+      <c r="D72" t="n">
         <v>0.2735154161934025</v>
+      </c>
+      <c r="E72" t="n">
+        <v>0.3260855209567263</v>
+      </c>
+      <c r="F72" t="n">
+        <v>0.3616956390907843</v>
       </c>
     </row>
     <row r="73">
@@ -1233,8 +2029,19 @@
       <c r="B73" t="n">
         <v>0.3510069218524295</v>
       </c>
-      <c r="C73" t="n">
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>80%&gt;gen/cap&gt;75%</t>
+        </is>
+      </c>
+      <c r="D73" t="n">
         <v>0.2874998238539221</v>
+      </c>
+      <c r="E73" t="n">
+        <v>0.3260855209567263</v>
+      </c>
+      <c r="F73" t="n">
+        <v>0.3428911998875694</v>
       </c>
     </row>
     <row r="74">
@@ -1242,10 +2049,21 @@
         <v>2378</v>
       </c>
       <c r="B74" t="n">
-        <v>0.4021462501649309</v>
-      </c>
-      <c r="C74" t="n">
+        <v>0.3341702609413204</v>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>30%&gt;gen/cap&gt;25%</t>
+        </is>
+      </c>
+      <c r="D74" t="n">
         <v>0.3015352332040474</v>
+      </c>
+      <c r="E74" t="n">
+        <v>0.317495714201756</v>
+      </c>
+      <c r="F74" t="n">
+        <v>0.3346443457314306</v>
       </c>
     </row>
     <row r="75">
@@ -1255,8 +2073,19 @@
       <c r="B75" t="n">
         <v>0.360039719292635</v>
       </c>
-      <c r="C75" t="n">
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>70%&gt;gen/cap&gt;65%</t>
+        </is>
+      </c>
+      <c r="D75" t="n">
         <v>0.2994914749965086</v>
+      </c>
+      <c r="E75" t="n">
+        <v>0.3261337513181191</v>
+      </c>
+      <c r="F75" t="n">
+        <v>0.3518757669663821</v>
       </c>
     </row>
     <row r="76">
@@ -1266,8 +2095,19 @@
       <c r="B76" t="n">
         <v>0.3576921311909673</v>
       </c>
-      <c r="C76" t="n">
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>60%&gt;gen/cap&gt;55%</t>
+        </is>
+      </c>
+      <c r="D76" t="n">
         <v>0.2950274441264135</v>
+      </c>
+      <c r="E76" t="n">
+        <v>0.3300662278897786</v>
+      </c>
+      <c r="F76" t="n">
+        <v>0.3455957022930549</v>
       </c>
     </row>
     <row r="77">
@@ -1277,8 +2117,19 @@
       <c r="B77" t="n">
         <v>0.3582742137454484</v>
       </c>
-      <c r="C77" t="n">
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>20%&gt;gen/cap&gt;15%</t>
+        </is>
+      </c>
+      <c r="D77" t="n">
         <v>0.2822159719845896</v>
+      </c>
+      <c r="E77" t="n">
+        <v>0.3027123616367527</v>
+      </c>
+      <c r="F77" t="n">
+        <v>0.3735316511005619</v>
       </c>
     </row>
     <row r="78">
@@ -1288,8 +2139,19 @@
       <c r="B78" t="n">
         <v>0.3682798786874736</v>
       </c>
-      <c r="C78" t="n">
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>5%&gt;gen/cap</t>
+        </is>
+      </c>
+      <c r="D78" t="n">
         <v>0.2833219127598758</v>
+      </c>
+      <c r="E78" t="n">
+        <v>0.1275782219601841</v>
+      </c>
+      <c r="F78" t="n">
+        <v>0.5586714557191558</v>
       </c>
     </row>
     <row r="79">
@@ -1299,8 +2161,19 @@
       <c r="B79" t="n">
         <v>0.3454269318322105</v>
       </c>
-      <c r="C79" t="n">
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>90%&gt;gen/cap&gt;85%</t>
+        </is>
+      </c>
+      <c r="D79" t="n">
         <v>0.1767351408063946</v>
+      </c>
+      <c r="E79" t="n">
+        <v>0.3261577166574556</v>
+      </c>
+      <c r="F79" t="n">
+        <v>0.3372390141666211</v>
       </c>
     </row>
     <row r="80">
@@ -1310,8 +2183,19 @@
       <c r="B80" t="n">
         <v>0.3323239723586519</v>
       </c>
-      <c r="C80" t="n">
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>95%&gt;gen/cap&gt;90%</t>
+        </is>
+      </c>
+      <c r="D80" t="n">
         <v>0.3007119184708865</v>
+      </c>
+      <c r="E80" t="n">
+        <v>0.3266645889845783</v>
+      </c>
+      <c r="F80" t="n">
+        <v>0.3236291823659397</v>
       </c>
     </row>
     <row r="81">
@@ -1321,8 +2205,19 @@
       <c r="B81" t="n">
         <v>0.3408509660557938</v>
       </c>
-      <c r="C81" t="n">
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>80%&gt;gen/cap&gt;75%</t>
+        </is>
+      </c>
+      <c r="D81" t="n">
         <v>0.3350687471037519</v>
+      </c>
+      <c r="E81" t="n">
+        <v>0.3260855209567263</v>
+      </c>
+      <c r="F81" t="n">
+        <v>0.3327352440909338</v>
       </c>
     </row>
     <row r="82">
@@ -1332,8 +2227,19 @@
       <c r="B82" t="n">
         <v>0.3350319360420932</v>
       </c>
-      <c r="C82" t="n">
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>50%&gt;gen/cap&gt;45%</t>
+        </is>
+      </c>
+      <c r="D82" t="n">
         <v>0.2990874840283987</v>
+      </c>
+      <c r="E82" t="n">
+        <v>0.3290786474885763</v>
+      </c>
+      <c r="F82" t="n">
+        <v>0.3239230875453831</v>
       </c>
     </row>
     <row r="83">
@@ -1343,8 +2249,19 @@
       <c r="B83" t="n">
         <v>0.2984522925637598</v>
       </c>
-      <c r="C83" t="n">
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>85%&gt;gen/cap&gt;80%</t>
+        </is>
+      </c>
+      <c r="D83" t="n">
         <v>0.2253424006096986</v>
+      </c>
+      <c r="E83" t="n">
+        <v>0.327678763896358</v>
+      </c>
+      <c r="F83" t="n">
+        <v>0.288743327659268</v>
       </c>
     </row>
     <row r="84">
@@ -1352,10 +2269,21 @@
         <v>2079</v>
       </c>
       <c r="B84" t="n">
-        <v>0.4920055140540828</v>
-      </c>
-      <c r="C84" t="n">
+        <v>0.3567019286784823</v>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>60%&gt;gen/cap&gt;55%</t>
+        </is>
+      </c>
+      <c r="D84" t="n">
         <v>0.332831843028485</v>
+      </c>
+      <c r="E84" t="n">
+        <v>0.3300662278897786</v>
+      </c>
+      <c r="F84" t="n">
+        <v>0.3446054997805699</v>
       </c>
     </row>
     <row r="85">
@@ -1365,8 +2293,19 @@
       <c r="B85" t="n">
         <v>0.4048803021393707</v>
       </c>
-      <c r="C85" t="n">
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>30%&gt;gen/cap&gt;25%</t>
+        </is>
+      </c>
+      <c r="D85" t="n">
         <v>0.2257864059858031</v>
+      </c>
+      <c r="E85" t="n">
+        <v>0.317495714201756</v>
+      </c>
+      <c r="F85" t="n">
+        <v>0.4053543869294809</v>
       </c>
     </row>
     <row r="86">
@@ -1376,8 +2315,19 @@
       <c r="B86" t="n">
         <v>0.3613718015950349</v>
       </c>
-      <c r="C86" t="n">
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>65%&gt;gen/cap&gt;60%</t>
+        </is>
+      </c>
+      <c r="D86" t="n">
         <v>0.2986295917733249</v>
+      </c>
+      <c r="E86" t="n">
+        <v>0.3252929965811113</v>
+      </c>
+      <c r="F86" t="n">
+        <v>0.3540486040057898</v>
       </c>
     </row>
     <row r="87">
@@ -1387,8 +2337,19 @@
       <c r="B87" t="n">
         <v>0.5213840596956788</v>
       </c>
-      <c r="C87" t="n">
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>100%&gt;gen/cap&gt;95%</t>
+        </is>
+      </c>
+      <c r="D87" t="n">
         <v>0.1869888518525323</v>
+      </c>
+      <c r="E87" t="n">
+        <v>0.3179697989918662</v>
+      </c>
+      <c r="F87" t="n">
+        <v>0.5213840596956788</v>
       </c>
     </row>
     <row r="88">
@@ -1396,10 +2357,21 @@
         <v>1723</v>
       </c>
       <c r="B88" t="n">
-        <v>0.3716312694452902</v>
-      </c>
-      <c r="C88" t="n">
+        <v>0.354343538904794</v>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>35%&gt;gen/cap&gt;30%</t>
+        </is>
+      </c>
+      <c r="D88" t="n">
         <v>0.2806189290612324</v>
+      </c>
+      <c r="E88" t="n">
+        <v>0.3228360886967814</v>
+      </c>
+      <c r="F88" t="n">
+        <v>0.3494772491998787</v>
       </c>
     </row>
     <row r="89">
@@ -1409,8 +2381,19 @@
       <c r="B89" t="n">
         <v>0.3744743974591479</v>
       </c>
-      <c r="C89" t="n">
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>50%&gt;gen/cap&gt;45%</t>
+        </is>
+      </c>
+      <c r="D89" t="n">
         <v>0.189875698102339</v>
+      </c>
+      <c r="E89" t="n">
+        <v>0.3290786474885763</v>
+      </c>
+      <c r="F89" t="n">
+        <v>0.3633655489624377</v>
       </c>
     </row>
     <row r="90">
@@ -1420,8 +2403,19 @@
       <c r="B90" t="n">
         <v>0.3940655355512691</v>
       </c>
-      <c r="C90" t="n">
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>85%&gt;gen/cap&gt;80%</t>
+        </is>
+      </c>
+      <c r="D90" t="n">
         <v>0.3432023137636835</v>
+      </c>
+      <c r="E90" t="n">
+        <v>0.327678763896358</v>
+      </c>
+      <c r="F90" t="n">
+        <v>0.3843565706467773</v>
       </c>
     </row>
     <row r="91">
@@ -1431,8 +2425,19 @@
       <c r="B91" t="n">
         <v>0.3729988994955625</v>
       </c>
-      <c r="C91" t="n">
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>30%&gt;gen/cap&gt;25%</t>
+        </is>
+      </c>
+      <c r="D91" t="n">
         <v>0.376989498882803</v>
+      </c>
+      <c r="E91" t="n">
+        <v>0.317495714201756</v>
+      </c>
+      <c r="F91" t="n">
+        <v>0.3734729842856726</v>
       </c>
     </row>
     <row r="92">
@@ -1440,10 +2445,21 @@
         <v>1619</v>
       </c>
       <c r="B92" t="n">
-        <v>0.4822602500308986</v>
-      </c>
-      <c r="C92" t="n">
+        <v>0.3474885087110839</v>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>20%&gt;gen/cap&gt;15%</t>
+        </is>
+      </c>
+      <c r="D92" t="n">
         <v>0.3129963387890729</v>
+      </c>
+      <c r="E92" t="n">
+        <v>0.3027123616367527</v>
+      </c>
+      <c r="F92" t="n">
+        <v>0.3627459460661974</v>
       </c>
     </row>
     <row r="93">
@@ -1453,8 +2469,19 @@
       <c r="B93" t="n">
         <v>0.4111931147911536</v>
       </c>
-      <c r="C93" t="n">
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>25%&gt;gen/cap&gt;20%</t>
+        </is>
+      </c>
+      <c r="D93" t="n">
         <v>0.2576834094500449</v>
+      </c>
+      <c r="E93" t="n">
+        <v>0.3119528493677421</v>
+      </c>
+      <c r="F93" t="n">
+        <v>0.4172100644152777</v>
       </c>
     </row>
     <row r="94">
@@ -1464,8 +2491,19 @@
       <c r="B94" t="n">
         <v>0.3850465353245314</v>
       </c>
-      <c r="C94" t="n">
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>85%&gt;gen/cap&gt;80%</t>
+        </is>
+      </c>
+      <c r="D94" t="n">
         <v>0.318426680414835</v>
+      </c>
+      <c r="E94" t="n">
+        <v>0.327678763896358</v>
+      </c>
+      <c r="F94" t="n">
+        <v>0.3753375704200396</v>
       </c>
     </row>
     <row r="95">
@@ -1475,8 +2513,19 @@
       <c r="B95" t="n">
         <v>0.3647835277017356</v>
       </c>
-      <c r="C95" t="n">
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>55%&gt;gen/cap&gt;50%</t>
+        </is>
+      </c>
+      <c r="D95" t="n">
         <v>0.3263599274711367</v>
+      </c>
+      <c r="E95" t="n">
+        <v>0.3299146687852249</v>
+      </c>
+      <c r="F95" t="n">
+        <v>0.3528386579083769</v>
       </c>
     </row>
     <row r="96">
@@ -1486,8 +2535,19 @@
       <c r="B96" t="n">
         <v>0.3309031813868305</v>
       </c>
-      <c r="C96" t="n">
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>30%&gt;gen/cap&gt;25%</t>
+        </is>
+      </c>
+      <c r="D96" t="n">
         <v>0.2175192469636241</v>
+      </c>
+      <c r="E96" t="n">
+        <v>0.317495714201756</v>
+      </c>
+      <c r="F96" t="n">
+        <v>0.3313772661769407</v>
       </c>
     </row>
     <row r="97">
@@ -1497,8 +2557,19 @@
       <c r="B97" t="n">
         <v>0.3189135236987325</v>
       </c>
-      <c r="C97" t="n">
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>100%&gt;gen/cap&gt;95%</t>
+        </is>
+      </c>
+      <c r="D97" t="n">
         <v>0.1819597408102214</v>
+      </c>
+      <c r="E97" t="n">
+        <v>0.3179697989918662</v>
+      </c>
+      <c r="F97" t="n">
+        <v>0.3189135236987325</v>
       </c>
     </row>
     <row r="98">
@@ -1508,8 +2579,19 @@
       <c r="B98" t="n">
         <v>0.3709580368288992</v>
       </c>
-      <c r="C98" t="n">
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>45%&gt;gen/cap&gt;40%</t>
+        </is>
+      </c>
+      <c r="D98" t="n">
         <v>0.3539739019315459</v>
+      </c>
+      <c r="E98" t="n">
+        <v>0.3259006427158213</v>
+      </c>
+      <c r="F98" t="n">
+        <v>0.3630271931049441</v>
       </c>
     </row>
     <row r="99">
@@ -1519,8 +2601,19 @@
       <c r="B99" t="n">
         <v>0.3091456705991906</v>
       </c>
-      <c r="C99" t="n">
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>95%&gt;gen/cap&gt;90%</t>
+        </is>
+      </c>
+      <c r="D99" t="n">
         <v>0.06304002232048303</v>
+      </c>
+      <c r="E99" t="n">
+        <v>0.3266645889845783</v>
+      </c>
+      <c r="F99" t="n">
+        <v>0.3004508806064785</v>
       </c>
     </row>
     <row r="100">
@@ -1530,8 +2623,19 @@
       <c r="B100" t="n">
         <v>0.3561356106057925</v>
       </c>
-      <c r="C100" t="n">
+      <c r="C100" t="inlineStr">
+        <is>
+          <t>40%&gt;gen/cap&gt;35%</t>
+        </is>
+      </c>
+      <c r="D100" t="n">
         <v>0.3316217407851156</v>
+      </c>
+      <c r="E100" t="n">
+        <v>0.3252845350267428</v>
+      </c>
+      <c r="F100" t="n">
+        <v>0.3488208745709158</v>
       </c>
     </row>
     <row r="101">
@@ -1541,8 +2645,19 @@
       <c r="B101" t="n">
         <v>0.2602492216789122</v>
       </c>
-      <c r="C101" t="n">
+      <c r="C101" t="inlineStr">
+        <is>
+          <t>35%&gt;gen/cap&gt;30%</t>
+        </is>
+      </c>
+      <c r="D101" t="n">
         <v>0.2192747352870803</v>
+      </c>
+      <c r="E101" t="n">
+        <v>0.3228360886967814</v>
+      </c>
+      <c r="F101" t="n">
+        <v>0.255382931973997</v>
       </c>
     </row>
     <row r="102">
@@ -1550,10 +2665,21 @@
         <v>1378</v>
       </c>
       <c r="B102" t="n">
-        <v>0.5667705677812378</v>
-      </c>
-      <c r="C102" t="n">
+        <v>0.3629443496312539</v>
+      </c>
+      <c r="C102" t="inlineStr">
+        <is>
+          <t>45%&gt;gen/cap&gt;40%</t>
+        </is>
+      </c>
+      <c r="D102" t="n">
         <v>0.1794564314696095</v>
+      </c>
+      <c r="E102" t="n">
+        <v>0.3259006427158213</v>
+      </c>
+      <c r="F102" t="n">
+        <v>0.3550135059072988</v>
       </c>
     </row>
     <row r="103">
@@ -1561,10 +2687,21 @@
         <v>1374</v>
       </c>
       <c r="B103" t="n">
-        <v>0.3139419296879841</v>
-      </c>
-      <c r="C103" t="n">
+        <v>0.3142709058074636</v>
+      </c>
+      <c r="C103" t="inlineStr">
+        <is>
+          <t>105%&gt;gen/cap&gt;100%</t>
+        </is>
+      </c>
+      <c r="D103" t="n">
         <v>0.1583872230727588</v>
+      </c>
+      <c r="E103" t="n">
+        <v>0.2915500913161409</v>
+      </c>
+      <c r="F103" t="n">
+        <v>0.3406906134831889</v>
       </c>
     </row>
     <row r="104">
@@ -1574,8 +2711,19 @@
       <c r="B104" t="n">
         <v>0.3147888834803775</v>
       </c>
-      <c r="C104" t="n">
+      <c r="C104" t="inlineStr">
+        <is>
+          <t>30%&gt;gen/cap&gt;25%</t>
+        </is>
+      </c>
+      <c r="D104" t="n">
         <v>0.2211515454740631</v>
+      </c>
+      <c r="E104" t="n">
+        <v>0.317495714201756</v>
+      </c>
+      <c r="F104" t="n">
+        <v>0.3152629682704878</v>
       </c>
     </row>
     <row r="105">
@@ -1583,10 +2731,21 @@
         <v>1356</v>
       </c>
       <c r="B105" t="n">
-        <v>0.404001646717537</v>
-      </c>
-      <c r="C105" t="n">
+        <v>0.3339595615357706</v>
+      </c>
+      <c r="C105" t="inlineStr">
+        <is>
+          <t>50%&gt;gen/cap&gt;45%</t>
+        </is>
+      </c>
+      <c r="D105" t="n">
         <v>0.3195114566958964</v>
+      </c>
+      <c r="E105" t="n">
+        <v>0.3290786474885763</v>
+      </c>
+      <c r="F105" t="n">
+        <v>0.3228507130390604</v>
       </c>
     </row>
     <row r="106">
@@ -1594,10 +2753,21 @@
         <v>1355</v>
       </c>
       <c r="B106" t="n">
-        <v>0.3487187858547596</v>
-      </c>
-      <c r="C106" t="n">
+        <v>0.3259858533473405</v>
+      </c>
+      <c r="C106" t="inlineStr">
+        <is>
+          <t>60%&gt;gen/cap&gt;55%</t>
+        </is>
+      </c>
+      <c r="D106" t="n">
         <v>0.3040080299850326</v>
+      </c>
+      <c r="E106" t="n">
+        <v>0.3300662278897786</v>
+      </c>
+      <c r="F106" t="n">
+        <v>0.3138894244494281</v>
       </c>
     </row>
     <row r="107">
@@ -1605,10 +2775,21 @@
         <v>1295</v>
       </c>
       <c r="B107" t="n">
-        <v>2.05177247605194</v>
-      </c>
-      <c r="C107" t="n">
+        <v>0.4290618842785497</v>
+      </c>
+      <c r="C107" t="inlineStr">
+        <is>
+          <t>30%&gt;gen/cap&gt;25%</t>
+        </is>
+      </c>
+      <c r="D107" t="n">
         <v>0.2749952266905087</v>
+      </c>
+      <c r="E107" t="n">
+        <v>0.317495714201756</v>
+      </c>
+      <c r="F107" t="n">
+        <v>0.4295359690686598</v>
       </c>
     </row>
     <row r="108">
@@ -1616,10 +2797,21 @@
         <v>1241</v>
       </c>
       <c r="B108" t="n">
-        <v>0.390066111243477</v>
-      </c>
-      <c r="C108" t="n">
+        <v>0.3539526385259697</v>
+      </c>
+      <c r="C108" t="inlineStr">
+        <is>
+          <t>50%&gt;gen/cap&gt;45%</t>
+        </is>
+      </c>
+      <c r="D108" t="n">
         <v>0.2325610711514961</v>
+      </c>
+      <c r="E108" t="n">
+        <v>0.3290786474885763</v>
+      </c>
+      <c r="F108" t="n">
+        <v>0.3428437900292595</v>
       </c>
     </row>
     <row r="109">
@@ -1629,8 +2821,19 @@
       <c r="B109" t="n">
         <v>0.3260176678836244</v>
       </c>
-      <c r="C109" t="n">
+      <c r="C109" t="inlineStr">
+        <is>
+          <t>65%&gt;gen/cap&gt;60%</t>
+        </is>
+      </c>
+      <c r="D109" t="n">
         <v>0.1521048992032321</v>
+      </c>
+      <c r="E109" t="n">
+        <v>0.3252929965811113</v>
+      </c>
+      <c r="F109" t="n">
+        <v>0.3186944702943793</v>
       </c>
     </row>
     <row r="110">
@@ -1638,10 +2841,21 @@
         <v>1081</v>
       </c>
       <c r="B110" t="n">
-        <v>0.5507934642717458</v>
-      </c>
-      <c r="C110" t="n">
+        <v>0.3524335072806861</v>
+      </c>
+      <c r="C110" t="inlineStr">
+        <is>
+          <t>50%&gt;gen/cap&gt;45%</t>
+        </is>
+      </c>
+      <c r="D110" t="n">
         <v>0.342973349438488</v>
+      </c>
+      <c r="E110" t="n">
+        <v>0.3290786474885763</v>
+      </c>
+      <c r="F110" t="n">
+        <v>0.3413246587839759</v>
       </c>
     </row>
     <row r="111">
@@ -1651,8 +2865,19 @@
       <c r="B111" t="n">
         <v>0.3474893300106217</v>
       </c>
-      <c r="C111" t="n">
+      <c r="C111" t="inlineStr">
+        <is>
+          <t>25%&gt;gen/cap&gt;20%</t>
+        </is>
+      </c>
+      <c r="D111" t="n">
         <v>0.3008380441315619</v>
+      </c>
+      <c r="E111" t="n">
+        <v>0.3119528493677421</v>
+      </c>
+      <c r="F111" t="n">
+        <v>0.3535062796347457</v>
       </c>
     </row>
     <row r="112">
@@ -1660,10 +2885,21 @@
         <v>1043</v>
       </c>
       <c r="B112" t="n">
-        <v>0.3453720536206965</v>
-      </c>
-      <c r="C112" t="n">
+        <v>0.3523532391946655</v>
+      </c>
+      <c r="C112" t="inlineStr">
+        <is>
+          <t>110%&gt;gen/cap&gt;105%</t>
+        </is>
+      </c>
+      <c r="D112" t="n">
         <v>0.3010690731983817</v>
+      </c>
+      <c r="E112" t="n">
+        <v>0.3429164079648739</v>
+      </c>
+      <c r="F112" t="n">
+        <v>0.3274066302216578</v>
       </c>
     </row>
     <row r="113">
@@ -1673,8 +2909,19 @@
       <c r="B113" t="n">
         <v>0.3046535248917526</v>
       </c>
-      <c r="C113" t="n">
+      <c r="C113" t="inlineStr">
+        <is>
+          <t>15%&gt;gen/cap&gt;10%</t>
+        </is>
+      </c>
+      <c r="D113" t="n">
         <v>0.2827103819132206</v>
+      </c>
+      <c r="E113" t="n">
+        <v>0.2861617054590648</v>
+      </c>
+      <c r="F113" t="n">
+        <v>0.336461618424554</v>
       </c>
     </row>
     <row r="114">
@@ -1682,10 +2929,21 @@
         <v>1010</v>
       </c>
       <c r="B114" t="n">
-        <v>0.5023904058892911</v>
-      </c>
-      <c r="C114" t="n">
+        <v>0.3570292035012889</v>
+      </c>
+      <c r="C114" t="inlineStr">
+        <is>
+          <t>65%&gt;gen/cap&gt;60%</t>
+        </is>
+      </c>
+      <c r="D114" t="n">
         <v>0.2494889898667585</v>
+      </c>
+      <c r="E114" t="n">
+        <v>0.3252929965811113</v>
+      </c>
+      <c r="F114" t="n">
+        <v>0.3497060059120438</v>
       </c>
     </row>
     <row r="115">
@@ -1695,8 +2953,19 @@
       <c r="B115" t="n">
         <v>0.2836355858900913</v>
       </c>
-      <c r="C115" t="n">
+      <c r="C115" t="inlineStr">
+        <is>
+          <t>90%&gt;gen/cap&gt;85%</t>
+        </is>
+      </c>
+      <c r="D115" t="n">
         <v>0.2248366001098001</v>
+      </c>
+      <c r="E115" t="n">
+        <v>0.3261577166574556</v>
+      </c>
+      <c r="F115" t="n">
+        <v>0.2754476682245019</v>
       </c>
     </row>
     <row r="116">
@@ -1706,8 +2975,19 @@
       <c r="B116" t="n">
         <v>0.3373614043107674</v>
       </c>
-      <c r="C116" t="n">
+      <c r="C116" t="inlineStr">
+        <is>
+          <t>35%&gt;gen/cap&gt;30%</t>
+        </is>
+      </c>
+      <c r="D116" t="n">
         <v>0.2351861726741784</v>
+      </c>
+      <c r="E116" t="n">
+        <v>0.3228360886967814</v>
+      </c>
+      <c r="F116" t="n">
+        <v>0.3324951146058522</v>
       </c>
     </row>
     <row r="117">
@@ -1717,8 +2997,19 @@
       <c r="B117" t="n">
         <v>0.3154158372992738</v>
       </c>
-      <c r="C117" t="n">
+      <c r="C117" t="inlineStr">
+        <is>
+          <t>35%&gt;gen/cap&gt;30%</t>
+        </is>
+      </c>
+      <c r="D117" t="n">
         <v>0.1414537313146478</v>
+      </c>
+      <c r="E117" t="n">
+        <v>0.3228360886967814</v>
+      </c>
+      <c r="F117" t="n">
+        <v>0.3105495475943585</v>
       </c>
     </row>
     <row r="118">
@@ -1728,8 +3019,19 @@
       <c r="B118" t="n">
         <v>0.3341057713080128</v>
       </c>
-      <c r="C118" t="n">
+      <c r="C118" t="inlineStr">
+        <is>
+          <t>25%&gt;gen/cap&gt;20%</t>
+        </is>
+      </c>
+      <c r="D118" t="n">
         <v>0.1099034620669631</v>
+      </c>
+      <c r="E118" t="n">
+        <v>0.3119528493677421</v>
+      </c>
+      <c r="F118" t="n">
+        <v>0.3401227209321369</v>
       </c>
     </row>
     <row r="119">
@@ -1737,10 +3039,21 @@
         <v>994</v>
       </c>
       <c r="B119" t="n">
-        <v>0.3193461637203914</v>
-      </c>
-      <c r="C119" t="n">
+        <v>0.3068712033032386</v>
+      </c>
+      <c r="C119" t="inlineStr">
+        <is>
+          <t>15%&gt;gen/cap&gt;10%</t>
+        </is>
+      </c>
+      <c r="D119" t="n">
         <v>0.3002334817384795</v>
+      </c>
+      <c r="E119" t="n">
+        <v>0.2861617054590648</v>
+      </c>
+      <c r="F119" t="n">
+        <v>0.33867929683604</v>
       </c>
     </row>
     <row r="120">
@@ -1750,8 +3063,19 @@
       <c r="B120" t="n">
         <v>0.377597647224074</v>
       </c>
-      <c r="C120" t="n">
+      <c r="C120" t="inlineStr">
+        <is>
+          <t>20%&gt;gen/cap&gt;15%</t>
+        </is>
+      </c>
+      <c r="D120" t="n">
         <v>0.3028253148388222</v>
+      </c>
+      <c r="E120" t="n">
+        <v>0.3027123616367527</v>
+      </c>
+      <c r="F120" t="n">
+        <v>0.3928550845791874</v>
       </c>
     </row>
     <row r="121">
@@ -1761,8 +3085,19 @@
       <c r="B121" t="n">
         <v>0.3200383648458848</v>
       </c>
-      <c r="C121" t="n">
+      <c r="C121" t="inlineStr">
+        <is>
+          <t>60%&gt;gen/cap&gt;55%</t>
+        </is>
+      </c>
+      <c r="D121" t="n">
         <v>0.3007083663699309</v>
+      </c>
+      <c r="E121" t="n">
+        <v>0.3300662278897786</v>
+      </c>
+      <c r="F121" t="n">
+        <v>0.3079419359479724</v>
       </c>
     </row>
     <row r="122">
@@ -1770,10 +3105,21 @@
         <v>988</v>
       </c>
       <c r="B122" t="n">
-        <v>0.4369362396923436</v>
-      </c>
-      <c r="C122" t="n">
+        <v>0.374447376636143</v>
+      </c>
+      <c r="C122" t="inlineStr">
+        <is>
+          <t>50%&gt;gen/cap&gt;45%</t>
+        </is>
+      </c>
+      <c r="D122" t="n">
         <v>0.219423550284241</v>
+      </c>
+      <c r="E122" t="n">
+        <v>0.3290786474885763</v>
+      </c>
+      <c r="F122" t="n">
+        <v>0.3633385281394328</v>
       </c>
     </row>
     <row r="123">
@@ -1781,10 +3127,21 @@
         <v>983</v>
       </c>
       <c r="B123" t="n">
-        <v>0.3643001584047057</v>
-      </c>
-      <c r="C123" t="n">
+        <v>0.3710993336921878</v>
+      </c>
+      <c r="C123" t="inlineStr">
+        <is>
+          <t>110%&gt;gen/cap&gt;105%</t>
+        </is>
+      </c>
+      <c r="D123" t="n">
         <v>0.3554259716397997</v>
+      </c>
+      <c r="E123" t="n">
+        <v>0.3429164079648739</v>
+      </c>
+      <c r="F123" t="n">
+        <v>0.34615272471918</v>
       </c>
     </row>
     <row r="124">
@@ -1794,8 +3151,19 @@
       <c r="B124" t="n">
         <v>0.3753025580695051</v>
       </c>
-      <c r="C124" t="n">
+      <c r="C124" t="inlineStr">
+        <is>
+          <t>80%&gt;gen/cap&gt;75%</t>
+        </is>
+      </c>
+      <c r="D124" t="n">
         <v>0.2080688625334745</v>
+      </c>
+      <c r="E124" t="n">
+        <v>0.3260855209567263</v>
+      </c>
+      <c r="F124" t="n">
+        <v>0.367186836104645</v>
       </c>
     </row>
     <row r="125">
@@ -1803,10 +3171,21 @@
         <v>892</v>
       </c>
       <c r="B125" t="n">
-        <v>0.3423287839730054</v>
-      </c>
-      <c r="C125" t="n">
+        <v>0.3446856235632145</v>
+      </c>
+      <c r="C125" t="inlineStr">
+        <is>
+          <t>105%&gt;gen/cap&gt;100%</t>
+        </is>
+      </c>
+      <c r="D125" t="n">
         <v>0.176354625030066</v>
+      </c>
+      <c r="E125" t="n">
+        <v>0.2915500913161409</v>
+      </c>
+      <c r="F125" t="n">
+        <v>0.3711053312389398</v>
       </c>
     </row>
     <row r="126">
@@ -1816,8 +3195,19 @@
       <c r="B126" t="n">
         <v>0.368209472500456</v>
       </c>
-      <c r="C126" t="n">
+      <c r="C126" t="inlineStr">
+        <is>
+          <t>100%&gt;gen/cap&gt;95%</t>
+        </is>
+      </c>
+      <c r="D126" t="n">
         <v>0.2468045397430277</v>
+      </c>
+      <c r="E126" t="n">
+        <v>0.3179697989918662</v>
+      </c>
+      <c r="F126" t="n">
+        <v>0.368209472500456</v>
       </c>
     </row>
     <row r="127">
@@ -1827,8 +3217,19 @@
       <c r="B127" t="n">
         <v>0.3217583741703381</v>
       </c>
-      <c r="C127" t="n">
+      <c r="C127" t="inlineStr">
+        <is>
+          <t>90%&gt;gen/cap&gt;85%</t>
+        </is>
+      </c>
+      <c r="D127" t="n">
         <v>0.3209856327912293</v>
+      </c>
+      <c r="E127" t="n">
+        <v>0.3261577166574556</v>
+      </c>
+      <c r="F127" t="n">
+        <v>0.3135704565047486</v>
       </c>
     </row>
     <row r="128">
@@ -1838,8 +3239,19 @@
       <c r="B128" t="n">
         <v>0.3490808065648447</v>
       </c>
-      <c r="C128" t="n">
+      <c r="C128" t="inlineStr">
+        <is>
+          <t>80%&gt;gen/cap&gt;75%</t>
+        </is>
+      </c>
+      <c r="D128" t="n">
         <v>0.1408378652040445</v>
+      </c>
+      <c r="E128" t="n">
+        <v>0.3260855209567263</v>
+      </c>
+      <c r="F128" t="n">
+        <v>0.3409650845999846</v>
       </c>
     </row>
     <row r="129">
@@ -1847,10 +3259,21 @@
         <v>874</v>
       </c>
       <c r="B129" t="n">
-        <v>0.3610796311341488</v>
-      </c>
-      <c r="C129" t="n">
+        <v>0.3426453863025116</v>
+      </c>
+      <c r="C129" t="inlineStr">
+        <is>
+          <t>55%&gt;gen/cap&gt;50%</t>
+        </is>
+      </c>
+      <c r="D129" t="n">
         <v>0.238954363544711</v>
+      </c>
+      <c r="E129" t="n">
+        <v>0.3299146687852249</v>
+      </c>
+      <c r="F129" t="n">
+        <v>0.3307005165091529</v>
       </c>
     </row>
     <row r="130">
@@ -1860,8 +3283,19 @@
       <c r="B130" t="n">
         <v>0.3032936621157706</v>
       </c>
-      <c r="C130" t="n">
+      <c r="C130" t="inlineStr">
+        <is>
+          <t>30%&gt;gen/cap&gt;25%</t>
+        </is>
+      </c>
+      <c r="D130" t="n">
         <v>0.1489170629055099</v>
+      </c>
+      <c r="E130" t="n">
+        <v>0.317495714201756</v>
+      </c>
+      <c r="F130" t="n">
+        <v>0.3037677469058808</v>
       </c>
     </row>
     <row r="131">
@@ -1871,8 +3305,19 @@
       <c r="B131" t="n">
         <v>0.3256974475820567</v>
       </c>
-      <c r="C131" t="n">
+      <c r="C131" t="inlineStr">
+        <is>
+          <t>85%&gt;gen/cap&gt;80%</t>
+        </is>
+      </c>
+      <c r="D131" t="n">
         <v>0.1879425499591285</v>
+      </c>
+      <c r="E131" t="n">
+        <v>0.327678763896358</v>
+      </c>
+      <c r="F131" t="n">
+        <v>0.3159884826775649</v>
       </c>
     </row>
     <row r="132">
@@ -1882,8 +3327,19 @@
       <c r="B132" t="n">
         <v>0.5887604521763219</v>
       </c>
-      <c r="C132" t="n">
+      <c r="C132" t="inlineStr">
+        <is>
+          <t>90%&gt;gen/cap&gt;85%</t>
+        </is>
+      </c>
+      <c r="D132" t="n">
         <v>0.2349389855258899</v>
+      </c>
+      <c r="E132" t="n">
+        <v>0.3261577166574556</v>
+      </c>
+      <c r="F132" t="n">
+        <v>0.5805725345107324</v>
       </c>
     </row>
     <row r="133">
@@ -1893,8 +3349,19 @@
       <c r="B133" t="n">
         <v>0.3167810529762386</v>
       </c>
-      <c r="C133" t="n">
+      <c r="C133" t="inlineStr">
+        <is>
+          <t>95%&gt;gen/cap&gt;90%</t>
+        </is>
+      </c>
+      <c r="D133" t="n">
         <v>0.1921135570225264</v>
+      </c>
+      <c r="E133" t="n">
+        <v>0.3266645889845783</v>
+      </c>
+      <c r="F133" t="n">
+        <v>0.3080862629835265</v>
       </c>
     </row>
     <row r="134">
@@ -1904,8 +3371,19 @@
       <c r="B134" t="n">
         <v>0.343957426640445</v>
       </c>
-      <c r="C134" t="n">
+      <c r="C134" t="inlineStr">
+        <is>
+          <t>20%&gt;gen/cap&gt;15%</t>
+        </is>
+      </c>
+      <c r="D134" t="n">
         <v>0.2946109943963943</v>
+      </c>
+      <c r="E134" t="n">
+        <v>0.3027123616367527</v>
+      </c>
+      <c r="F134" t="n">
+        <v>0.3592148639955585</v>
       </c>
     </row>
     <row r="135">
@@ -1915,8 +3393,19 @@
       <c r="B135" t="n">
         <v>0.3452912417166399</v>
       </c>
-      <c r="C135" t="n">
+      <c r="C135" t="inlineStr">
+        <is>
+          <t>85%&gt;gen/cap&gt;80%</t>
+        </is>
+      </c>
+      <c r="D135" t="n">
         <v>0.2813944014617442</v>
+      </c>
+      <c r="E135" t="n">
+        <v>0.327678763896358</v>
+      </c>
+      <c r="F135" t="n">
+        <v>0.3355822768121481</v>
       </c>
     </row>
     <row r="136">
@@ -1924,10 +3413,21 @@
         <v>727</v>
       </c>
       <c r="B136" t="n">
-        <v>0.3493932630422841</v>
-      </c>
-      <c r="C136" t="n">
+        <v>0.3412049189465816</v>
+      </c>
+      <c r="C136" t="inlineStr">
+        <is>
+          <t>50%&gt;gen/cap&gt;45%</t>
+        </is>
+      </c>
+      <c r="D136" t="n">
         <v>0.2340505526158381</v>
+      </c>
+      <c r="E136" t="n">
+        <v>0.3290786474885763</v>
+      </c>
+      <c r="F136" t="n">
+        <v>0.3300960704498714</v>
       </c>
     </row>
     <row r="137">
@@ -1937,8 +3437,19 @@
       <c r="B137" t="n">
         <v>0.3920208048396226</v>
       </c>
-      <c r="C137" t="n">
+      <c r="C137" t="inlineStr">
+        <is>
+          <t>80%&gt;gen/cap&gt;75%</t>
+        </is>
+      </c>
+      <c r="D137" t="n">
         <v>0.3084731658007794</v>
+      </c>
+      <c r="E137" t="n">
+        <v>0.3260855209567263</v>
+      </c>
+      <c r="F137" t="n">
+        <v>0.3839050828747625</v>
       </c>
     </row>
     <row r="138">
@@ -1948,8 +3459,19 @@
       <c r="B138" t="n">
         <v>0.3770303255745312</v>
       </c>
-      <c r="C138" t="n">
+      <c r="C138" t="inlineStr">
+        <is>
+          <t>95%&gt;gen/cap&gt;90%</t>
+        </is>
+      </c>
+      <c r="D138" t="n">
         <v>0.417394023590101</v>
+      </c>
+      <c r="E138" t="n">
+        <v>0.3266645889845783</v>
+      </c>
+      <c r="F138" t="n">
+        <v>0.3683355355818191</v>
       </c>
     </row>
     <row r="139">
@@ -1959,8 +3481,19 @@
       <c r="B139" t="n">
         <v>0.3532671931796519</v>
       </c>
-      <c r="C139" t="n">
+      <c r="C139" t="inlineStr">
+        <is>
+          <t>85%&gt;gen/cap&gt;80%</t>
+        </is>
+      </c>
+      <c r="D139" t="n">
         <v>0.2801051729978689</v>
+      </c>
+      <c r="E139" t="n">
+        <v>0.327678763896358</v>
+      </c>
+      <c r="F139" t="n">
+        <v>0.3435582282751601</v>
       </c>
     </row>
     <row r="140">
@@ -1970,8 +3503,19 @@
       <c r="B140" t="n">
         <v>0.3692435881529905</v>
       </c>
-      <c r="C140" t="n">
+      <c r="C140" t="inlineStr">
+        <is>
+          <t>90%&gt;gen/cap&gt;85%</t>
+        </is>
+      </c>
+      <c r="D140" t="n">
         <v>0.2522407233200708</v>
+      </c>
+      <c r="E140" t="n">
+        <v>0.3261577166574556</v>
+      </c>
+      <c r="F140" t="n">
+        <v>0.3610556704874011</v>
       </c>
     </row>
     <row r="141">
@@ -1981,8 +3525,19 @@
       <c r="B141" t="n">
         <v>0.4209821611508353</v>
       </c>
-      <c r="C141" t="n">
+      <c r="C141" t="inlineStr">
+        <is>
+          <t>85%&gt;gen/cap&gt;80%</t>
+        </is>
+      </c>
+      <c r="D141" t="n">
         <v>0.2431552076022918</v>
+      </c>
+      <c r="E141" t="n">
+        <v>0.327678763896358</v>
+      </c>
+      <c r="F141" t="n">
+        <v>0.4112731962463435</v>
       </c>
     </row>
     <row r="142">
@@ -1992,8 +3547,19 @@
       <c r="B142" t="n">
         <v>0.3350241609741931</v>
       </c>
-      <c r="C142" t="n">
+      <c r="C142" t="inlineStr">
+        <is>
+          <t>95%&gt;gen/cap&gt;90%</t>
+        </is>
+      </c>
+      <c r="D142" t="n">
         <v>0.2930353422789901</v>
+      </c>
+      <c r="E142" t="n">
+        <v>0.3266645889845783</v>
+      </c>
+      <c r="F142" t="n">
+        <v>0.326329370981481</v>
       </c>
     </row>
     <row r="143">
@@ -2001,10 +3567,21 @@
         <v>642</v>
       </c>
       <c r="B143" t="n">
-        <v>0.2647797501931667</v>
-      </c>
-      <c r="C143" t="n">
+        <v>0.2762891919450974</v>
+      </c>
+      <c r="C143" t="inlineStr">
+        <is>
+          <t>105%&gt;gen/cap&gt;100%</t>
+        </is>
+      </c>
+      <c r="D143" t="n">
         <v>0.1664603001366493</v>
+      </c>
+      <c r="E143" t="n">
+        <v>0.2915500913161409</v>
+      </c>
+      <c r="F143" t="n">
+        <v>0.3027088996208226</v>
       </c>
     </row>
     <row r="144">
@@ -2014,8 +3591,19 @@
       <c r="B144" t="n">
         <v>0.3958268962092519</v>
       </c>
-      <c r="C144" t="n">
+      <c r="C144" t="inlineStr">
+        <is>
+          <t>5%&gt;gen/cap</t>
+        </is>
+      </c>
+      <c r="D144" t="n">
         <v>0.3236362580725322</v>
+      </c>
+      <c r="E144" t="n">
+        <v>0.1275782219601841</v>
+      </c>
+      <c r="F144" t="n">
+        <v>0.586218473240934</v>
       </c>
     </row>
     <row r="145">
@@ -2025,8 +3613,19 @@
       <c r="B145" t="n">
         <v>0.3519491089564129</v>
       </c>
-      <c r="C145" t="n">
+      <c r="C145" t="inlineStr">
+        <is>
+          <t>60%&gt;gen/cap&gt;55%</t>
+        </is>
+      </c>
+      <c r="D145" t="n">
         <v>0.3319633994983702</v>
+      </c>
+      <c r="E145" t="n">
+        <v>0.3300662278897786</v>
+      </c>
+      <c r="F145" t="n">
+        <v>0.3398526800585004</v>
       </c>
     </row>
     <row r="146">
@@ -2036,8 +3635,19 @@
       <c r="B146" t="n">
         <v>0.3505273733544978</v>
       </c>
-      <c r="C146" t="n">
+      <c r="C146" t="inlineStr">
+        <is>
+          <t>100%&gt;gen/cap&gt;95%</t>
+        </is>
+      </c>
+      <c r="D146" t="n">
         <v>0.2801632709223243</v>
+      </c>
+      <c r="E146" t="n">
+        <v>0.3179697989918662</v>
+      </c>
+      <c r="F146" t="n">
+        <v>0.3505273733544978</v>
       </c>
     </row>
     <row r="147">
@@ -2047,8 +3657,19 @@
       <c r="B147" t="n">
         <v>0.2758229919721963</v>
       </c>
-      <c r="C147" t="n">
+      <c r="C147" t="inlineStr">
+        <is>
+          <t>70%&gt;gen/cap&gt;65%</t>
+        </is>
+      </c>
+      <c r="D147" t="n">
         <v>0.1188680437542776</v>
+      </c>
+      <c r="E147" t="n">
+        <v>0.3261337513181191</v>
+      </c>
+      <c r="F147" t="n">
+        <v>0.2676590396459434</v>
       </c>
     </row>
   </sheetData>

</xml_diff>